<commit_message>
changed error algo remove titles small fixes
</commit_message>
<xml_diff>
--- a/results/radial_T_left.xlsx
+++ b/results/radial_T_left.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,2954 +413,3259 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I101"/>
+  <dimension ref="A1:J101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Radius_mm</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>T_K</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>T_err</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Intercept_b</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Intercept_b_err</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Partition_func</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Partition_func_err</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Electron_concentration</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Electron_concentration_err</t>
         </is>
       </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Electron_concentration_rel_err</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>6006.4947406527</v>
+        <v>5018.986087816946</v>
       </c>
       <c r="C2" t="n">
-        <v>411.8764859001662</v>
+        <v>288.4342615278226</v>
       </c>
       <c r="D2" t="n">
-        <v>42.43857615168042</v>
+        <v>41.18898708825403</v>
       </c>
       <c r="E2" t="n">
-        <v>0.7306523061380352</v>
+        <v>0.7328259265877131</v>
       </c>
       <c r="F2" t="n">
-        <v>11.12462145899258</v>
+        <v>8.923834472811341</v>
       </c>
       <c r="G2" t="n">
-        <v>1.154023742841807</v>
+        <v>0.4889950496281588</v>
       </c>
       <c r="H2" t="n">
-        <v>2.261330641177269e+21</v>
+        <v>5.199249953187356e+20</v>
       </c>
       <c r="I2" t="n">
-        <v>1.668815974511158e+21</v>
+        <v>3.820781940206094e+20</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.7348717554661506</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.02411111111111111</v>
+        <v>0.01002020202020202</v>
       </c>
       <c r="B3" t="n">
-        <v>6003.147369100879</v>
+        <v>5019.188211072533</v>
       </c>
       <c r="C3" t="n">
-        <v>411.6060635634352</v>
+        <v>286.6276682731414</v>
       </c>
       <c r="D3" t="n">
-        <v>42.44256663679519</v>
+        <v>41.1878176990027</v>
       </c>
       <c r="E3" t="n">
-        <v>0.730987107327171</v>
+        <v>0.7281772577549274</v>
       </c>
       <c r="F3" t="n">
-        <v>11.11524941232332</v>
+        <v>8.924177230688409</v>
       </c>
       <c r="G3" t="n">
-        <v>1.151561701030751</v>
+        <v>0.4859899275421474</v>
       </c>
       <c r="H3" t="n">
-        <v>2.26845977849248e+21</v>
+        <v>5.193373025656841e+20</v>
       </c>
       <c r="I3" t="n">
-        <v>1.674786384820108e+21</v>
+        <v>3.792256874220627e+20</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.7302107619625484</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0.04822222222222222</v>
+        <v>0.02004040404040404</v>
       </c>
       <c r="B4" t="n">
-        <v>5999.595274753598</v>
+        <v>5019.3930095429</v>
       </c>
       <c r="C4" t="n">
-        <v>411.3922916813083</v>
+        <v>284.9517520736008</v>
       </c>
       <c r="D4" t="n">
-        <v>42.44659698949805</v>
+        <v>41.18661037743617</v>
       </c>
       <c r="E4" t="n">
-        <v>0.7314728382516134</v>
+        <v>0.7238605218790688</v>
       </c>
       <c r="F4" t="n">
-        <v>11.1053194973945</v>
+        <v>8.924524539198373</v>
       </c>
       <c r="G4" t="n">
-        <v>1.149155722179618</v>
+        <v>0.4832064323486406</v>
       </c>
       <c r="H4" t="n">
-        <v>2.275586185860476e+21</v>
+        <v>5.187308608170727e+20</v>
       </c>
       <c r="I4" t="n">
-        <v>1.68110259746641e+21</v>
+        <v>3.765377210258676e+20</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.7258826290627257</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>0.07233333333333333</v>
+        <v>0.03006060606060606</v>
       </c>
       <c r="B5" t="n">
-        <v>5995.845879943843</v>
+        <v>5019.595695242954</v>
       </c>
       <c r="C5" t="n">
-        <v>411.2127367909225</v>
+        <v>283.408056791919</v>
       </c>
       <c r="D5" t="n">
-        <v>42.45061145039275</v>
+        <v>41.1853737029818</v>
       </c>
       <c r="E5" t="n">
-        <v>0.7320682955861502</v>
+        <v>0.719880946324328</v>
       </c>
       <c r="F5" t="n">
-        <v>11.09485481167102</v>
+        <v>8.92486826475624</v>
       </c>
       <c r="G5" t="n">
-        <v>1.146748819988057</v>
+        <v>0.4806458980580458</v>
       </c>
       <c r="H5" t="n">
-        <v>2.282586858967956e+21</v>
+        <v>5.181097101949688e+20</v>
       </c>
       <c r="I5" t="n">
-        <v>1.687582076843276e+21</v>
+        <v>3.740195575908123e+20</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.7218925841981726</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0.09644444444444444</v>
+        <v>0.04008080808080808</v>
       </c>
       <c r="B6" t="n">
-        <v>5991.905625697917</v>
+        <v>5019.791450895215</v>
       </c>
       <c r="C6" t="n">
-        <v>411.0448160347862</v>
+        <v>281.9981348898792</v>
       </c>
       <c r="D6" t="n">
-        <v>42.4545551765254</v>
+        <v>41.18411630127167</v>
       </c>
       <c r="E6" t="n">
-        <v>0.7327320857754868</v>
+        <v>0.7162437572438347</v>
       </c>
       <c r="F6" t="n">
-        <v>11.08387619517378</v>
+        <v>8.925200237957904</v>
       </c>
       <c r="G6" t="n">
-        <v>1.144280113435997</v>
+        <v>0.4783096953042156</v>
       </c>
       <c r="H6" t="n">
-        <v>2.289338932399447e+21</v>
+        <v>5.174778951810213e+20</v>
       </c>
       <c r="I6" t="n">
-        <v>1.69404034674735e+21</v>
+        <v>3.716763526601635e+20</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.7182458538255934</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>0.1205555555555556</v>
+        <v>0.0501010101010101</v>
       </c>
       <c r="B7" t="n">
-        <v>5987.779900884829</v>
+        <v>5019.975427126391</v>
       </c>
       <c r="C7" t="n">
-        <v>410.8657211590268</v>
+        <v>280.7235521480305</v>
       </c>
       <c r="D7" t="n">
-        <v>42.45837419354639</v>
+        <v>41.1828468492555</v>
       </c>
       <c r="E7" t="n">
-        <v>0.733422477618684</v>
+        <v>0.7129541987295451</v>
       </c>
       <c r="F7" t="n">
-        <v>11.0724014388194</v>
+        <v>8.925512234969425</v>
       </c>
       <c r="G7" t="n">
-        <v>1.141688265248869</v>
+        <v>0.4761992323525943</v>
       </c>
       <c r="H7" t="n">
-        <v>2.295719530272531e+21</v>
+        <v>5.168394650626537e+20</v>
       </c>
       <c r="I7" t="n">
-        <v>1.700290607497066e+21</v>
+        <v>3.695131778008937e+20</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.7149476825576769</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>0.1446666666666667</v>
+        <v>0.06012121212121212</v>
       </c>
       <c r="B8" t="n">
-        <v>5983.472969066938</v>
+        <v>5020.142739489424</v>
       </c>
       <c r="C8" t="n">
-        <v>410.6523203738994</v>
+        <v>279.5858925419573</v>
       </c>
       <c r="D8" t="n">
-        <v>42.46201532806555</v>
+        <v>41.18157408078308</v>
       </c>
       <c r="E8" t="n">
-        <v>0.7340972163702133</v>
+        <v>0.7100175526315191</v>
       </c>
       <c r="F8" t="n">
-        <v>11.06044510078839</v>
+        <v>8.92579611450263</v>
       </c>
       <c r="G8" t="n">
-        <v>1.138913048943721</v>
+        <v>0.4743159760940072</v>
       </c>
       <c r="H8" t="n">
-        <v>2.301605755380832e+21</v>
+        <v>5.161984839128037e+20</v>
       </c>
       <c r="I8" t="n">
-        <v>1.706143411192344e+21</v>
+        <v>3.675350513904395e+20</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.7120033530600673</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>0.1687777777777778</v>
+        <v>0.07014141414141414</v>
       </c>
       <c r="B9" t="n">
-        <v>5978.987890676918</v>
+        <v>5020.288465301522</v>
       </c>
       <c r="C9" t="n">
-        <v>410.3810363716158</v>
+        <v>278.5867632830231</v>
       </c>
       <c r="D9" t="n">
-        <v>42.46542612175998</v>
+        <v>41.18030679267662</v>
       </c>
       <c r="E9" t="n">
-        <v>0.7347132958062434</v>
+        <v>0.7074391590816577</v>
       </c>
       <c r="F9" t="n">
-        <v>11.04801832999133</v>
+        <v>8.926043389346887</v>
       </c>
       <c r="G9" t="n">
-        <v>1.135891661976477</v>
+        <v>0.4726613935262697</v>
       </c>
       <c r="H9" t="n">
-        <v>2.306874696632854e+21</v>
+        <v>5.15559008389384e+20</v>
       </c>
       <c r="I9" t="n">
-        <v>1.711406202625309e+21</v>
+        <v>3.657469469417526e+20</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.7094182062386087</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>0.1928888888888889</v>
+        <v>0.08016161616161616</v>
       </c>
       <c r="B10" t="n">
-        <v>5974.326437838429</v>
+        <v>5020.407640287426</v>
       </c>
       <c r="C10" t="n">
-        <v>410.0276981916822</v>
+        <v>277.7278000316922</v>
       </c>
       <c r="D10" t="n">
-        <v>42.46855472872569</v>
+        <v>41.17905385131709</v>
       </c>
       <c r="E10" t="n">
-        <v>0.735226683532195</v>
+        <v>0.7052244377608532</v>
       </c>
       <c r="F10" t="n">
-        <v>11.03512942209174</v>
+        <v>8.926245611421718</v>
       </c>
       <c r="G10" t="n">
-        <v>1.13255929844694</v>
+        <v>0.4712370080913481</v>
       </c>
       <c r="H10" t="n">
-        <v>2.311403609118733e+21</v>
+        <v>5.149251132057369e+20</v>
       </c>
       <c r="I10" t="n">
-        <v>1.715883104858535e+21</v>
+        <v>3.641538365587316e+20</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.7071976627662262</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>0.217</v>
+        <v>0.09018181818181817</v>
       </c>
       <c r="B11" t="n">
-        <v>5969.488998762085</v>
+        <v>5020.495255016331</v>
       </c>
       <c r="C11" t="n">
-        <v>409.5673638681463</v>
+        <v>277.0106722940487</v>
       </c>
       <c r="D11" t="n">
-        <v>42.47134979751065</v>
+        <v>41.17782419977021</v>
       </c>
       <c r="E11" t="n">
-        <v>0.7355919933434218</v>
+        <v>0.7033789099584032</v>
       </c>
       <c r="F11" t="n">
-        <v>11.02178208816803</v>
+        <v>8.92639428047446</v>
       </c>
       <c r="G11" t="n">
-        <v>1.128850169733883</v>
+        <v>0.4700443886340545</v>
       </c>
       <c r="H11" t="n">
-        <v>2.315069638378526e+21</v>
+        <v>5.143008895574619e+20</v>
       </c>
       <c r="I11" t="n">
-        <v>1.719374373747513e+21</v>
+        <v>3.627607155765664e+20</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0.7053472450508679</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>0.2411111111111111</v>
+        <v>0.1002020202020202</v>
       </c>
       <c r="B12" t="n">
-        <v>5964.474468158673</v>
+        <v>5020.5462511195</v>
       </c>
       <c r="C12" t="n">
-        <v>408.9741098497338</v>
+        <v>276.4370890137138</v>
       </c>
       <c r="D12" t="n">
-        <v>42.47376033924351</v>
+        <v>41.17662686548159</v>
       </c>
       <c r="E12" t="n">
-        <v>0.7357620966169455</v>
+        <v>0.7019082214804386</v>
       </c>
       <c r="F12" t="n">
-        <v>11.00797648064912</v>
+        <v>8.926480813212123</v>
       </c>
       <c r="G12" t="n">
-        <v>1.124694586784033</v>
+        <v>0.4690851470942469</v>
       </c>
       <c r="H12" t="n">
-        <v>2.317750145244437e+21</v>
+        <v>5.136904476564794e+20</v>
       </c>
       <c r="I12" t="n">
-        <v>1.721676152207145e+21</v>
+        <v>3.615726310368726e+20</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0.7038726000968336</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>0.2652222222222222</v>
+        <v>0.1102222222222222</v>
       </c>
       <c r="B13" t="n">
-        <v>5959.280119481388</v>
+        <v>5020.55551727454</v>
       </c>
       <c r="C13" t="n">
-        <v>408.2207820041907</v>
+        <v>276.0088043727026</v>
       </c>
       <c r="D13" t="n">
-        <v>42.47573558330357</v>
+        <v>41.17547096857279</v>
       </c>
       <c r="E13" t="n">
-        <v>0.735687662405986</v>
+        <v>0.7008181664716333</v>
       </c>
       <c r="F13" t="n">
-        <v>10.99370836824857</v>
+        <v>8.926496536487303</v>
       </c>
       <c r="G13" t="n">
-        <v>1.120018845814102</v>
+        <v>0.4683609396678091</v>
       </c>
       <c r="H13" t="n">
-        <v>2.319322674142516e+21</v>
+        <v>5.130979212730385e+20</v>
       </c>
       <c r="I13" t="n">
-        <v>1.722580010644667e+21</v>
+        <v>3.605947125165986e+20</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0.7027795232963197</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>0.2893333333333333</v>
+        <v>0.1202424242424242</v>
       </c>
       <c r="B14" t="n">
-        <v>5953.963806337249</v>
+        <v>5020.517884940696</v>
       </c>
       <c r="C14" t="n">
-        <v>407.2954483187228</v>
+        <v>275.7276238173119</v>
       </c>
       <c r="D14" t="n">
-        <v>42.47714691165108</v>
+        <v>41.17436573077449</v>
       </c>
       <c r="E14" t="n">
-        <v>0.7353314466501545</v>
+        <v>0.700114712225511</v>
       </c>
       <c r="F14" t="n">
-        <v>10.97913946387026</v>
+        <v>8.92643268006162</v>
       </c>
       <c r="G14" t="n">
-        <v>1.114822823166878</v>
+        <v>0.4678734679849667</v>
       </c>
       <c r="H14" t="n">
-        <v>2.319520394770234e+21</v>
+        <v>5.125274728947542e+20</v>
       </c>
       <c r="I14" t="n">
-        <v>1.721800982032883e+21</v>
+        <v>3.598322043989862e+20</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0.7020739832084602</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>0.3134444444444444</v>
+        <v>0.1302626262626262</v>
       </c>
       <c r="B15" t="n">
-        <v>5949.040597603348</v>
+        <v>5020.428123828103</v>
       </c>
       <c r="C15" t="n">
-        <v>406.3358274702575</v>
+        <v>275.595410327079</v>
       </c>
       <c r="D15" t="n">
-        <v>42.47729029928717</v>
+        <v>41.17332048503629</v>
       </c>
       <c r="E15" t="n">
-        <v>0.7348136484013141</v>
+        <v>0.6998040250685102</v>
       </c>
       <c r="F15" t="n">
-        <v>10.96567884884916</v>
+        <v>8.926280368917716</v>
       </c>
       <c r="G15" t="n">
-        <v>1.109743669532215</v>
+        <v>0.4676244803031152</v>
       </c>
       <c r="H15" t="n">
-        <v>2.317008829218669e+21</v>
+        <v>5.11983299531499e+20</v>
       </c>
       <c r="I15" t="n">
-        <v>1.718640968905124e+21</v>
+        <v>3.592904997177524e+20</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0.7017621474109188</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>0.3375555555555556</v>
+        <v>0.1402828282828283</v>
       </c>
       <c r="B16" t="n">
-        <v>5944.658859082729</v>
+        <v>5020.280937082243</v>
       </c>
       <c r="C16" t="n">
-        <v>405.4312526818402</v>
+        <v>275.6140909470751</v>
       </c>
       <c r="D16" t="n">
-        <v>42.47591407904746</v>
+        <v>41.17234468585696</v>
       </c>
       <c r="E16" t="n">
-        <v>0.7342590563308534</v>
+        <v>0.6998924974140085</v>
       </c>
       <c r="F16" t="n">
-        <v>10.95372375678434</v>
+        <v>8.926030615088004</v>
       </c>
       <c r="G16" t="n">
-        <v>1.105096980741525</v>
+        <v>0.467615772710952</v>
       </c>
       <c r="H16" t="n">
-        <v>2.31129971367525e+21</v>
+        <v>5.114696391992213e+20</v>
       </c>
       <c r="I16" t="n">
-        <v>1.71303753564148e+21</v>
+        <v>3.589751757290748e+20</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0.7018504095201069</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>0.3616666666666667</v>
+        <v>0.1503030303030303</v>
       </c>
       <c r="B17" t="n">
-        <v>5940.86123817285</v>
+        <v>5020.070956162771</v>
       </c>
       <c r="C17" t="n">
-        <v>404.6486970713824</v>
+        <v>275.7856636065774</v>
       </c>
       <c r="D17" t="n">
-        <v>42.47289481715958</v>
+        <v>41.17144792038439</v>
       </c>
       <c r="E17" t="n">
-        <v>0.7337790229040024</v>
+        <v>0.7003867760955583</v>
       </c>
       <c r="F17" t="n">
-        <v>10.94338121902258</v>
+        <v>8.925674308964798</v>
       </c>
       <c r="G17" t="n">
-        <v>1.101083506653085</v>
+        <v>0.4678491903407955</v>
       </c>
       <c r="H17" t="n">
-        <v>2.302156061990218e+21</v>
+        <v>5.109907781211715e+20</v>
       </c>
       <c r="I17" t="n">
-        <v>1.705080836959662e+21</v>
+        <v>3.588920313926219e+20</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0.702345417489154</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>0.3857777777777778</v>
+        <v>0.1603232323232323</v>
       </c>
       <c r="B18" t="n">
-        <v>5937.527052429062</v>
+        <v>5019.788039188816</v>
       </c>
       <c r="C18" t="n">
-        <v>404.0353663992649</v>
+        <v>276.1198275134107</v>
       </c>
       <c r="D18" t="n">
-        <v>42.46844045762778</v>
+        <v>41.17064817353861</v>
       </c>
       <c r="E18" t="n">
-        <v>0.7334899067280676</v>
+        <v>0.7013144665413285</v>
       </c>
       <c r="F18" t="n">
-        <v>10.93431549563819</v>
+        <v>8.925194452198548</v>
       </c>
       <c r="G18" t="n">
-        <v>1.097766368953396</v>
+        <v>0.4683382964888926</v>
       </c>
       <c r="H18" t="n">
-        <v>2.290025558775176e+21</v>
+        <v>5.105548286089647e+20</v>
       </c>
       <c r="I18" t="n">
-        <v>1.695372116226934e+21</v>
+        <v>3.590603557319657e+20</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0.7032748210613263</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>0.4098888888888889</v>
+        <v>0.1703434343434343</v>
       </c>
       <c r="B19" t="n">
-        <v>5933.910665243898</v>
+        <v>5019.409155852218</v>
       </c>
       <c r="C19" t="n">
-        <v>403.5566370896991</v>
+        <v>276.6471476614858</v>
       </c>
       <c r="D19" t="n">
-        <v>42.46403385157861</v>
+        <v>41.16998610031116</v>
       </c>
       <c r="E19" t="n">
-        <v>0.7335140717426495</v>
+        <v>0.7027598843793079</v>
       </c>
       <c r="F19" t="n">
-        <v>10.92449763699467</v>
+        <v>8.924551920997763</v>
       </c>
       <c r="G19" t="n">
-        <v>1.094681908398566</v>
+        <v>0.4691283607542771</v>
       </c>
       <c r="H19" t="n">
-        <v>2.277909359960172e+21</v>
+        <v>5.101801849150425e+20</v>
       </c>
       <c r="I19" t="n">
-        <v>1.686397392279388e+21</v>
+        <v>3.595357600489022e+20</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0.7047230972107899</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>0.434</v>
+        <v>0.1803636363636363</v>
       </c>
       <c r="B20" t="n">
-        <v>5929.886386432377</v>
+        <v>5019.04125218368</v>
       </c>
       <c r="C20" t="n">
-        <v>403.2654744443954</v>
+        <v>277.5261552610632</v>
       </c>
       <c r="D20" t="n">
-        <v>42.45989640259451</v>
+        <v>41.169273821197</v>
       </c>
       <c r="E20" t="n">
-        <v>0.7339800560202736</v>
+        <v>0.7050961635377003</v>
       </c>
       <c r="F20" t="n">
-        <v>10.91359134534973</v>
+        <v>8.923928009721955</v>
       </c>
       <c r="G20" t="n">
-        <v>1.091910388311735</v>
+        <v>0.470517307046343</v>
       </c>
       <c r="H20" t="n">
-        <v>2.266239372940122e+21</v>
+        <v>5.097812825478285e+20</v>
       </c>
       <c r="I20" t="n">
-        <v>1.678756992150015e+21</v>
+        <v>3.60448376041467e+20</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0.7070647518480616</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>0.4581111111111111</v>
+        <v>0.1903838383838384</v>
       </c>
       <c r="B21" t="n">
-        <v>5925.417573934613</v>
+        <v>5018.780895498178</v>
       </c>
       <c r="C21" t="n">
-        <v>403.2305392180064</v>
+        <v>278.8811487782948</v>
       </c>
       <c r="D21" t="n">
-        <v>42.4560665354791</v>
+        <v>41.16834160983211</v>
       </c>
       <c r="E21" t="n">
-        <v>0.7350238937100929</v>
+        <v>0.7086122394774669</v>
       </c>
       <c r="F21" t="n">
-        <v>10.90150354839498</v>
+        <v>8.923486700763148</v>
       </c>
       <c r="G21" t="n">
-        <v>1.089616560064458</v>
+        <v>0.4727422786026879</v>
       </c>
       <c r="H21" t="n">
-        <v>2.255076104770069e+21</v>
+        <v>5.092810937003691e+20</v>
       </c>
       <c r="I21" t="n">
-        <v>1.67278975665823e+21</v>
+        <v>3.618899637545126e+20</v>
+      </c>
+      <c r="J21" t="n">
+        <v>0.7105898259938691</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>0.4822222222222222</v>
+        <v>0.2004040404040404</v>
       </c>
       <c r="B22" t="n">
-        <v>5920.465088220356</v>
+        <v>5018.609467053686</v>
       </c>
       <c r="C22" t="n">
-        <v>403.5242401810368</v>
+        <v>280.6241388960001</v>
       </c>
       <c r="D22" t="n">
-        <v>42.45258590527985</v>
+        <v>41.16722229502176</v>
       </c>
       <c r="E22" t="n">
-        <v>0.7367903724319674</v>
+        <v>0.7130897363538719</v>
       </c>
       <c r="F22" t="n">
-        <v>10.88813582016149</v>
+        <v>8.923196153721143</v>
       </c>
       <c r="G22" t="n">
-        <v>1.087972939806795</v>
+        <v>0.475648998442937</v>
       </c>
       <c r="H22" t="n">
-        <v>2.244485033538987e+21</v>
+        <v>5.08694803194908e+20</v>
       </c>
       <c r="I22" t="n">
-        <v>1.66885366422448e+21</v>
+        <v>3.637571117822818e+20</v>
+      </c>
+      <c r="J22" t="n">
+        <v>0.7150792764102746</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>0.5063333333333333</v>
+        <v>0.2104242424242424</v>
       </c>
       <c r="B23" t="n">
-        <v>5914.986937342482</v>
+        <v>5018.508247071353</v>
       </c>
       <c r="C23" t="n">
-        <v>404.2232604497676</v>
+        <v>282.6665457501169</v>
       </c>
       <c r="D23" t="n">
-        <v>42.44949992011551</v>
+        <v>41.16594890976845</v>
       </c>
       <c r="E23" t="n">
-        <v>0.7394344561529538</v>
+        <v>0.7183086401253846</v>
       </c>
       <c r="F23" t="n">
-        <v>10.87338388568957</v>
+        <v>8.923024600123107</v>
       </c>
       <c r="G23" t="n">
-        <v>1.087160101564466</v>
+        <v>0.4790823304110702</v>
       </c>
       <c r="H23" t="n">
-        <v>2.234537662258387e+21</v>
+        <v>5.080376834803623e+20</v>
       </c>
       <c r="I23" t="n">
-        <v>1.667330543505683e+21</v>
+        <v>3.659458525418675e+20</v>
+      </c>
+      <c r="J23" t="n">
+        <v>0.7203124186279239</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>0.5304444444444445</v>
+        <v>0.2204444444444444</v>
       </c>
       <c r="B24" t="n">
-        <v>5908.937857451634</v>
+        <v>5018.458888883636</v>
       </c>
       <c r="C24" t="n">
-        <v>405.409169204923</v>
+        <v>284.9193591636673</v>
       </c>
       <c r="D24" t="n">
-        <v>42.44685836497739</v>
+        <v>41.16455347840908</v>
       </c>
       <c r="E24" t="n">
-        <v>0.743122968298658</v>
+        <v>0.7240477032752392</v>
       </c>
       <c r="F24" t="n">
-        <v>10.85713716792088</v>
+        <v>8.92294094495443</v>
       </c>
       <c r="G24" t="n">
-        <v>1.087364071056731</v>
+        <v>0.4828865507398113</v>
       </c>
       <c r="H24" t="n">
-        <v>2.225312818919535e+21</v>
+        <v>5.073244898531044e+20</v>
       </c>
       <c r="I24" t="n">
-        <v>1.668631746711678e+21</v>
+        <v>3.6835173924781e+20</v>
+      </c>
+      <c r="J24" t="n">
+        <v>0.7260673328710507</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>0.5545555555555556</v>
+        <v>0.2304646464646465</v>
       </c>
       <c r="B25" t="n">
-        <v>5902.354994189691</v>
+        <v>5018.447116983846</v>
       </c>
       <c r="C25" t="n">
-        <v>407.1103200240408</v>
+        <v>287.2936022697878</v>
       </c>
       <c r="D25" t="n">
-        <v>42.4446065882373</v>
+        <v>41.1630565475789</v>
       </c>
       <c r="E25" t="n">
-        <v>0.7479066966264106</v>
+        <v>0.7300846435624848</v>
       </c>
       <c r="F25" t="n">
-        <v>10.83950743451143</v>
+        <v>8.922920993244125</v>
       </c>
       <c r="G25" t="n">
-        <v>1.088669805127289</v>
+        <v>0.4869070946888854</v>
       </c>
       <c r="H25" t="n">
-        <v>2.216702230938782e+21</v>
+        <v>5.065644956251062e+20</v>
       </c>
       <c r="I25" t="n">
-        <v>1.672768342042542e+21</v>
+        <v>3.708665427124785e+20</v>
+      </c>
+      <c r="J25" t="n">
+        <v>0.7321210742470711</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>0.5786666666666667</v>
+        <v>0.2404848484848485</v>
       </c>
       <c r="B26" t="n">
-        <v>5895.708365966439</v>
+        <v>5018.456238971403</v>
       </c>
       <c r="C26" t="n">
-        <v>409.013992364076</v>
+        <v>289.6996210249336</v>
       </c>
       <c r="D26" t="n">
-        <v>42.4421377455708</v>
+        <v>41.16148574952248</v>
       </c>
       <c r="E26" t="n">
-        <v>0.7530991246603593</v>
+        <v>0.736196260497226</v>
       </c>
       <c r="F26" t="n">
-        <v>10.82176021616065</v>
+        <v>8.922936453726832</v>
       </c>
       <c r="G26" t="n">
-        <v>1.090460206472962</v>
+        <v>0.4909874619112323</v>
       </c>
       <c r="H26" t="n">
-        <v>2.207615897421741e+21</v>
+        <v>5.057702860548823e+20</v>
       </c>
       <c r="I26" t="n">
-        <v>1.67736971560873e+21</v>
+        <v>3.733847964122232e+20</v>
+      </c>
+      <c r="J26" t="n">
+        <v>0.7382497681402074</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>0.6027777777777777</v>
+        <v>0.2505050505050505</v>
       </c>
       <c r="B27" t="n">
-        <v>5889.04357204854</v>
+        <v>5018.468568920513</v>
       </c>
       <c r="C27" t="n">
-        <v>411.0206002255164</v>
+        <v>292.0472315678095</v>
       </c>
       <c r="D27" t="n">
-        <v>42.43938107029865</v>
+        <v>41.15987176237992</v>
       </c>
       <c r="E27" t="n">
-        <v>0.7585077401138383</v>
+        <v>0.7421584554238037</v>
       </c>
       <c r="F27" t="n">
-        <v>10.80401822846965</v>
+        <v>8.92295735125205</v>
       </c>
       <c r="G27" t="n">
-        <v>1.092489764065214</v>
+        <v>0.4949698138070019</v>
       </c>
       <c r="H27" t="n">
-        <v>2.197929233782487e+21</v>
+        <v>5.049558203203427e+20</v>
       </c>
       <c r="I27" t="n">
-        <v>1.681895620760376e+21</v>
+        <v>3.758025805293316e+20</v>
+      </c>
+      <c r="J27" t="n">
+        <v>0.7442286342811602</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>0.6268888888888888</v>
+        <v>0.2605252525252525</v>
       </c>
       <c r="B28" t="n">
-        <v>5882.318397425583</v>
+        <v>5018.466610335087</v>
       </c>
       <c r="C28" t="n">
-        <v>413.0812912960402</v>
+        <v>294.245823922553</v>
       </c>
       <c r="D28" t="n">
-        <v>42.43637697562762</v>
+        <v>41.15824492441489</v>
       </c>
       <c r="E28" t="n">
-        <v>0.7640546662597082</v>
+        <v>0.7477461624253621</v>
       </c>
       <c r="F28" t="n">
-        <v>10.78617026546561</v>
+        <v>8.922954031725915</v>
       </c>
       <c r="G28" t="n">
-        <v>1.094602159721442</v>
+        <v>0.498695475891049</v>
       </c>
       <c r="H28" t="n">
-        <v>2.18771632220202e+21</v>
+        <v>5.041348193187235e+20</v>
       </c>
       <c r="I28" t="n">
-        <v>1.686214382972843e+21</v>
+        <v>3.780163800903712e+20</v>
+      </c>
+      <c r="J28" t="n">
+        <v>0.7498319211539763</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>0.651</v>
+        <v>0.2705454545454545</v>
       </c>
       <c r="B29" t="n">
-        <v>5875.488117551822</v>
+        <v>5018.433017032564</v>
       </c>
       <c r="C29" t="n">
-        <v>415.1446435771858</v>
+        <v>296.204305773466</v>
       </c>
       <c r="D29" t="n">
-        <v>42.43316884169331</v>
+        <v>41.15663530332077</v>
       </c>
       <c r="E29" t="n">
-        <v>0.7696574847235278</v>
+        <v>0.7527331917073437</v>
       </c>
       <c r="F29" t="n">
-        <v>10.76809930132489</v>
+        <v>8.922897095814793</v>
       </c>
       <c r="G29" t="n">
-        <v>1.096641184148683</v>
+        <v>0.5020048561695559</v>
       </c>
       <c r="H29" t="n">
-        <v>2.17705555883701e+21</v>
+        <v>5.033207943772262e+20</v>
       </c>
       <c r="I29" t="n">
-        <v>1.690192200598898e+21</v>
+        <v>3.799230188981329e+20</v>
+      </c>
+      <c r="J29" t="n">
+        <v>0.7548327490983617</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>0.6751111111111111</v>
+        <v>0.2805656565656566</v>
       </c>
       <c r="B30" t="n">
-        <v>5868.505227456985</v>
+        <v>5018.350522755065</v>
       </c>
       <c r="C30" t="n">
-        <v>417.1563850132339</v>
+        <v>297.831020002247</v>
       </c>
       <c r="D30" t="n">
-        <v>42.42980336078141</v>
+        <v>41.15507282264036</v>
       </c>
       <c r="E30" t="n">
-        <v>0.7752287431843329</v>
+        <v>0.7568919849679718</v>
       </c>
       <c r="F30" t="n">
-        <v>10.74968283967836</v>
+        <v>8.922757279646126</v>
       </c>
       <c r="G30" t="n">
-        <v>1.098436920010482</v>
+        <v>0.5047373405627862</v>
       </c>
       <c r="H30" t="n">
-        <v>2.166030171210677e+21</v>
+        <v>5.025271050240585e+20</v>
       </c>
       <c r="I30" t="n">
-        <v>1.693692952940165e+21</v>
+        <v>3.814195126544786e+20</v>
+      </c>
+      <c r="J30" t="n">
+        <v>0.7590028654001023</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>0.6992222222222222</v>
+        <v>0.2905858585858586</v>
       </c>
       <c r="B31" t="n">
-        <v>5861.319120826475</v>
+        <v>5018.201838882454</v>
       </c>
       <c r="C31" t="n">
-        <v>419.0590560027373</v>
+        <v>299.0336356382699</v>
       </c>
       <c r="D31" t="n">
-        <v>42.42633095786103</v>
+        <v>41.15358744638002</v>
       </c>
       <c r="E31" t="n">
-        <v>0.7806753357486745</v>
+        <v>0.7599932822207627</v>
       </c>
       <c r="F31" t="n">
-        <v>10.73079184643325</v>
+        <v>8.922505281446478</v>
       </c>
       <c r="G31" t="n">
-        <v>1.099814014075909</v>
+        <v>0.5067311644406373</v>
       </c>
       <c r="H31" t="n">
-        <v>2.15472859907337e+21</v>
+        <v>5.017670458910839e+20</v>
       </c>
       <c r="I31" t="n">
-        <v>1.696578170309628e+21</v>
+        <v>3.824028428420531e+20</v>
+      </c>
+      <c r="J31" t="n">
+        <v>0.7621123108293154</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>0.7233333333333334</v>
+        <v>0.3006060606060606</v>
       </c>
       <c r="B32" t="n">
-        <v>5853.875710206113</v>
+        <v>5017.96951935838</v>
       </c>
       <c r="C32" t="n">
-        <v>420.7916043340493</v>
+        <v>299.7190115380697</v>
       </c>
       <c r="D32" t="n">
-        <v>42.4228063010934</v>
+        <v>41.15220942344257</v>
       </c>
       <c r="E32" t="n">
-        <v>0.7858977305030485</v>
+        <v>0.7618056979839876</v>
       </c>
       <c r="F32" t="n">
-        <v>10.7112900234887</v>
+        <v>8.922111562938463</v>
       </c>
       <c r="G32" t="n">
-        <v>1.100588954085825</v>
+        <v>0.5078232685864035</v>
       </c>
       <c r="H32" t="n">
-        <v>2.143245127118781e+21</v>
+        <v>5.010539648786076e+20</v>
       </c>
       <c r="I32" t="n">
-        <v>1.698706505269292e+21</v>
+        <v>3.82769652131777e+20</v>
+      </c>
+      <c r="J32" t="n">
+        <v>0.7639289956013263</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>0.7474444444444445</v>
+        <v>0.3106262626262626</v>
       </c>
       <c r="B33" t="n">
-        <v>5846.113546077089</v>
+        <v>5017.635923817293</v>
       </c>
       <c r="C33" t="n">
-        <v>422.2884050496507</v>
+        <v>299.7928182638078</v>
       </c>
       <c r="D33" t="n">
-        <v>42.41929613490016</v>
+        <v>41.15096936165648</v>
       </c>
       <c r="E33" t="n">
-        <v>0.7907890145240262</v>
+        <v>0.7620946199875572</v>
       </c>
       <c r="F33" t="n">
-        <v>10.69102415488184</v>
+        <v>8.921546497460854</v>
       </c>
       <c r="G33" t="n">
-        <v>1.100562237009703</v>
+        <v>0.5078488621286626</v>
       </c>
       <c r="H33" t="n">
-        <v>2.131694336391358e+21</v>
+        <v>5.004013180917803e+20</v>
       </c>
       <c r="I33" t="n">
-        <v>1.699943639612465e+21</v>
+        <v>3.824154928691555e+20</v>
+      </c>
+      <c r="J33" t="n">
+        <v>0.7642175970428107</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>0.7715555555555556</v>
+        <v>0.3206464646464646</v>
       </c>
       <c r="B34" t="n">
-        <v>5837.760049130101</v>
+        <v>5017.211793421587</v>
       </c>
       <c r="C34" t="n">
-        <v>423.4492469608178</v>
+        <v>299.1128896822489</v>
       </c>
       <c r="D34" t="n">
-        <v>42.41630863009087</v>
+        <v>41.14984796769125</v>
       </c>
       <c r="E34" t="n">
-        <v>0.7952338309552588</v>
+        <v>0.7604947539457307</v>
       </c>
       <c r="F34" t="n">
-        <v>10.66929535593388</v>
+        <v>8.920828078252262</v>
       </c>
       <c r="G34" t="n">
-        <v>1.099338634360591</v>
+        <v>0.5065708983790613</v>
       </c>
       <c r="H34" t="n">
-        <v>2.121015789218201e+21</v>
+        <v>4.9980023528003e+20</v>
       </c>
       <c r="I34" t="n">
-        <v>1.700802864695949e+21</v>
+        <v>3.811535802812539e+20</v>
+      </c>
+      <c r="J34" t="n">
+        <v>0.76261184644641</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>0.7956666666666666</v>
+        <v>0.3306666666666667</v>
       </c>
       <c r="B35" t="n">
-        <v>5828.620921295167</v>
+        <v>5016.708481771551</v>
       </c>
       <c r="C35" t="n">
-        <v>424.1802664207307</v>
+        <v>297.6740742560091</v>
       </c>
       <c r="D35" t="n">
-        <v>42.41418755366474</v>
+        <v>41.14882483742852</v>
       </c>
       <c r="E35" t="n">
-        <v>0.7991067549446628</v>
+        <v>0.7569884346129037</v>
       </c>
       <c r="F35" t="n">
-        <v>10.64561888259407</v>
+        <v>8.919975826536605</v>
       </c>
       <c r="G35" t="n">
-        <v>1.096590065536253</v>
+        <v>0.503985110568912</v>
       </c>
       <c r="H35" t="n">
-        <v>2.111824899481888e+21</v>
+        <v>4.992414364288401e+20</v>
       </c>
       <c r="I35" t="n">
-        <v>1.701536484298095e+21</v>
+        <v>3.789712188480158e+20</v>
+      </c>
+      <c r="J35" t="n">
+        <v>0.7590940799282651</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>0.8197777777777777</v>
+        <v>0.3406868686868686</v>
       </c>
       <c r="B36" t="n">
-        <v>5818.596827673186</v>
+        <v>5016.303471787873</v>
       </c>
       <c r="C36" t="n">
-        <v>424.3551542492234</v>
+        <v>295.9062588611631</v>
       </c>
       <c r="D36" t="n">
-        <v>42.41305657891596</v>
+        <v>41.14758702332557</v>
       </c>
       <c r="E36" t="n">
-        <v>0.8021930827549126</v>
+        <v>0.7526143762257395</v>
       </c>
       <c r="F36" t="n">
-        <v>10.61976476534932</v>
+        <v>8.919290197285536</v>
       </c>
       <c r="G36" t="n">
-        <v>1.091951189257926</v>
+        <v>0.5008728173267548</v>
       </c>
       <c r="H36" t="n">
-        <v>2.104314815111952e+21</v>
+        <v>4.98585524185039e+20</v>
       </c>
       <c r="I36" t="n">
-        <v>1.701877166590103e+21</v>
+        <v>3.76285738902522e+20</v>
+      </c>
+      <c r="J36" t="n">
+        <v>0.7547065060053205</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>0.8438888888888889</v>
+        <v>0.3507070707070707</v>
       </c>
       <c r="B37" t="n">
-        <v>5807.572979923498</v>
+        <v>5016.00372348991</v>
       </c>
       <c r="C37" t="n">
-        <v>423.7599094407917</v>
+        <v>293.9245790386428</v>
       </c>
       <c r="D37" t="n">
-        <v>42.41306170909421</v>
+        <v>41.14612164188683</v>
       </c>
       <c r="E37" t="n">
-        <v>0.8041118792652907</v>
+        <v>0.7476634792413088</v>
       </c>
       <c r="F37" t="n">
-        <v>10.59147076568496</v>
+        <v>8.918782762384364</v>
       </c>
       <c r="G37" t="n">
-        <v>1.084842196101819</v>
+        <v>0.497430816629847</v>
       </c>
       <c r="H37" t="n">
-        <v>2.098719103402439e+21</v>
+        <v>4.978271173518608e+20</v>
       </c>
       <c r="I37" t="n">
-        <v>1.701240662378312e+21</v>
+        <v>3.732413287413155e+20</v>
+      </c>
+      <c r="J37" t="n">
+        <v>0.7497408552726771</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>0.868</v>
+        <v>0.3607272727272727</v>
       </c>
       <c r="B38" t="n">
-        <v>5795.6181922437</v>
+        <v>5015.781767411633</v>
       </c>
       <c r="C38" t="n">
-        <v>422.4607535482086</v>
+        <v>291.7811301939991</v>
       </c>
       <c r="D38" t="n">
-        <v>42.41410955398203</v>
+        <v>41.14447644772911</v>
       </c>
       <c r="E38" t="n">
-        <v>0.8049572166941611</v>
+        <v>0.7422768229484094</v>
       </c>
       <c r="F38" t="n">
-        <v>10.5609512272671</v>
+        <v>8.918407236957789</v>
       </c>
       <c r="G38" t="n">
-        <v>1.075498748159135</v>
+        <v>0.4937388570981567</v>
       </c>
       <c r="H38" t="n">
-        <v>2.09486554611846e+21</v>
+        <v>4.96987841884283e+20</v>
       </c>
       <c r="I38" t="n">
-        <v>1.699718389769451e+21</v>
+        <v>3.699271865704091e+20</v>
+      </c>
+      <c r="J38" t="n">
+        <v>0.7443385036701597</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>0.8921111111111111</v>
+        <v>0.3707474747474747</v>
       </c>
       <c r="B39" t="n">
-        <v>5782.824582980143</v>
+        <v>5015.61003145679</v>
       </c>
       <c r="C39" t="n">
-        <v>420.5607237275872</v>
+        <v>289.5283436796926</v>
       </c>
       <c r="D39" t="n">
-        <v>42.41607479082597</v>
+        <v>41.14269940067225</v>
       </c>
       <c r="E39" t="n">
-        <v>0.8048864888418354</v>
+        <v>0.7365962849754933</v>
       </c>
       <c r="F39" t="n">
-        <v>10.52847859985636</v>
+        <v>8.918116681360925</v>
       </c>
       <c r="G39" t="n">
-        <v>1.064265555198258</v>
+        <v>0.4898773196382321</v>
       </c>
       <c r="H39" t="n">
-        <v>2.092532574231975e+21</v>
+        <v>4.960892925801622e+20</v>
       </c>
       <c r="I39" t="n">
-        <v>1.697481625796497e+21</v>
+        <v>3.664322030464783e+20</v>
+      </c>
+      <c r="J39" t="n">
+        <v>0.7386416286887854</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>0.9162222222222223</v>
+        <v>0.3807676767676768</v>
       </c>
       <c r="B40" t="n">
-        <v>5769.291104735295</v>
+        <v>5015.460870859371</v>
       </c>
       <c r="C40" t="n">
-        <v>418.1706108874694</v>
+        <v>287.2189620236715</v>
       </c>
       <c r="D40" t="n">
-        <v>42.41882101810438</v>
+        <v>41.14083860046343</v>
       </c>
       <c r="E40" t="n">
-        <v>0.804071306046314</v>
+        <v>0.7307643936263979</v>
       </c>
       <c r="F40" t="n">
-        <v>10.49433960727727</v>
+        <v>8.917864320424327</v>
       </c>
       <c r="G40" t="n">
-        <v>1.051508192998458</v>
+        <v>0.4859272553263433</v>
       </c>
       <c r="H40" t="n">
-        <v>2.091483266594039e+21</v>
+        <v>4.951530158438533e+20</v>
       </c>
       <c r="I40" t="n">
-        <v>1.694708428654976e+21</v>
+        <v>3.628446945505189e+20</v>
+      </c>
+      <c r="J40" t="n">
+        <v>0.7327930618218068</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>0.9403333333333334</v>
+        <v>0.3907878787878787</v>
       </c>
       <c r="B41" t="n">
-        <v>5755.124680658017</v>
+        <v>5015.306581285862</v>
       </c>
       <c r="C41" t="n">
-        <v>415.4103390175237</v>
+        <v>284.9060343214804</v>
       </c>
       <c r="D41" t="n">
-        <v>42.42219859038887</v>
+        <v>41.13894225644704</v>
       </c>
       <c r="E41" t="n">
-        <v>0.8027009755648213</v>
+        <v>0.7249242672263355</v>
       </c>
       <c r="F41" t="n">
-        <v>10.45883617096028</v>
+        <v>8.917603281906436</v>
       </c>
       <c r="G41" t="n">
-        <v>1.03760867268405</v>
+        <v>0.4819704237366605</v>
       </c>
       <c r="H41" t="n">
-        <v>2.091459702446285e+21</v>
+        <v>4.942004587667823e+20</v>
       </c>
       <c r="I41" t="n">
-        <v>1.691590454750203e+21</v>
+        <v>3.592522175624931e+20</v>
+      </c>
+      <c r="J41" t="n">
+        <v>0.7269362283858735</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>0.9644444444444444</v>
+        <v>0.4008080808080808</v>
       </c>
       <c r="B42" t="n">
-        <v>5740.441433765595</v>
+        <v>5015.119394842566</v>
       </c>
       <c r="C42" t="n">
-        <v>412.4104445739482</v>
+        <v>282.6429321539188</v>
       </c>
       <c r="D42" t="n">
-        <v>42.42604226848768</v>
+        <v>41.13705869267381</v>
       </c>
       <c r="E42" t="n">
-        <v>0.800986206969627</v>
+        <v>0.7192196416854489</v>
       </c>
       <c r="F42" t="n">
-        <v>10.42228767852725</v>
+        <v>8.917286586029871</v>
       </c>
       <c r="G42" t="n">
-        <v>1.022976227362355</v>
+        <v>0.4780893320355956</v>
       </c>
       <c r="H42" t="n">
-        <v>2.092177299711112e+21</v>
+        <v>4.932529590083171e+20</v>
       </c>
       <c r="I42" t="n">
-        <v>1.68834024170959e+21</v>
+        <v>3.557415192970976e+20</v>
+      </c>
+      <c r="J42" t="n">
+        <v>0.7212151752973046</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>0.9885555555555555</v>
+        <v>0.4108282828282828</v>
       </c>
       <c r="B43" t="n">
-        <v>5725.368011521659</v>
+        <v>5014.871458761338</v>
       </c>
       <c r="C43" t="n">
-        <v>409.3136539462056</v>
+        <v>280.4833863888616</v>
       </c>
       <c r="D43" t="n">
-        <v>42.43016868112424</v>
+        <v>41.13523638891032</v>
       </c>
       <c r="E43" t="n">
-        <v>0.7991630223379407</v>
+        <v>0.7137949874056401</v>
       </c>
       <c r="F43" t="n">
-        <v>10.38503190293692</v>
+        <v>8.91686723719037</v>
       </c>
       <c r="G43" t="n">
-        <v>1.008044328855035</v>
+        <v>0.4743673112604557</v>
       </c>
       <c r="H43" t="n">
-        <v>2.093318648576778e+21</v>
+        <v>4.923317670504016e+20</v>
       </c>
       <c r="I43" t="n">
-        <v>1.685197632985326e+21</v>
+        <v>3.52398617102046e+20</v>
+      </c>
+      <c r="J43" t="n">
+        <v>0.7157746883027554</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>1.012666666666667</v>
+        <v>0.4208484848484848</v>
       </c>
       <c r="B44" t="n">
-        <v>5710.043002616762</v>
+        <v>5014.534707043461</v>
       </c>
       <c r="C44" t="n">
-        <v>406.2765486598322</v>
+        <v>278.4815353776537</v>
       </c>
       <c r="D44" t="n">
-        <v>42.43437360622876</v>
+        <v>41.13352431370939</v>
       </c>
       <c r="E44" t="n">
-        <v>0.7974968190535054</v>
+        <v>0.708795716975416</v>
       </c>
       <c r="F44" t="n">
-        <v>10.34742756601887</v>
+        <v>8.916297830445647</v>
       </c>
       <c r="G44" t="n">
-        <v>0.9932670647358781</v>
+        <v>0.4708884658184853</v>
       </c>
       <c r="H44" t="n">
-        <v>2.094527554595353e+21</v>
+        <v>4.914581940118102e+20</v>
       </c>
       <c r="I44" t="n">
-        <v>1.682435801319231e+21</v>
+        <v>3.493090712135436e+20</v>
+      </c>
+      <c r="J44" t="n">
+        <v>0.7107604990001436</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>1.036777777777778</v>
+        <v>0.4308686868686868</v>
       </c>
       <c r="B45" t="n">
-        <v>5694.618435794673</v>
+        <v>5014.078779594018</v>
       </c>
       <c r="C45" t="n">
-        <v>403.4712967916975</v>
+        <v>276.6917824676983</v>
       </c>
       <c r="D45" t="n">
-        <v>42.43842909615872</v>
+        <v>41.13197782409686</v>
       </c>
       <c r="E45" t="n">
-        <v>0.796286490234403</v>
+        <v>0.7043684870794149</v>
       </c>
       <c r="F45" t="n">
-        <v>10.30985661722114</v>
+        <v>8.915526911839933</v>
       </c>
       <c r="G45" t="n">
-        <v>0.9791395313286034</v>
+        <v>0.4677367522033126</v>
       </c>
       <c r="H45" t="n">
-        <v>2.09540311650314e+21</v>
+        <v>4.906563197436743e+20</v>
       </c>
       <c r="I45" t="n">
-        <v>1.68036659491778e+21</v>
+        <v>3.46560165718987e+20</v>
+      </c>
+      <c r="J45" t="n">
+        <v>0.7063195800678463</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>1.060888888888889</v>
+        <v>0.4408888888888889</v>
       </c>
       <c r="B46" t="n">
-        <v>5679.261341312044</v>
+        <v>5013.474343760392</v>
       </c>
       <c r="C46" t="n">
-        <v>401.0874145512673</v>
+        <v>275.1692765472849</v>
       </c>
       <c r="D46" t="n">
-        <v>42.44208049273711</v>
+        <v>41.13064911498353</v>
       </c>
       <c r="E46" t="n">
-        <v>0.7958684520337804</v>
+        <v>0.7006615917341388</v>
       </c>
       <c r="F46" t="n">
-        <v>10.27272556087556</v>
+        <v>8.914505405879874</v>
       </c>
       <c r="G46" t="n">
-        <v>0.9661827441500619</v>
+        <v>0.4649976906173114</v>
       </c>
       <c r="H46" t="n">
-        <v>2.095494027698247e+21</v>
+        <v>4.89948670325718e+20</v>
       </c>
       <c r="I46" t="n">
-        <v>1.679342821773005e+21</v>
+        <v>3.442382048419439e+20</v>
+      </c>
+      <c r="J46" t="n">
+        <v>0.7026005491822118</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>1.085</v>
+        <v>0.4509090909090909</v>
       </c>
       <c r="B47" t="n">
-        <v>5664.163354419645</v>
+        <v>5012.692595343234</v>
       </c>
       <c r="C47" t="n">
-        <v>399.3207488060687</v>
+        <v>273.9701264626496</v>
       </c>
       <c r="D47" t="n">
-        <v>42.44503234879885</v>
+        <v>41.12958847972713</v>
       </c>
       <c r="E47" t="n">
-        <v>0.7965926591773049</v>
+        <v>0.6978258105716006</v>
       </c>
       <c r="F47" t="n">
-        <v>10.23648829456673</v>
+        <v>8.913184645734425</v>
       </c>
       <c r="G47" t="n">
-        <v>0.9549254524726105</v>
+        <v>0.4627584457099669</v>
       </c>
       <c r="H47" t="n">
-        <v>2.094275009400431e+21</v>
+        <v>4.89356775846854e+20</v>
       </c>
       <c r="I47" t="n">
-        <v>1.679684574796893e+21</v>
+        <v>3.424296143095889e+20</v>
+      </c>
+      <c r="J47" t="n">
+        <v>0.6997545169717923</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>1.109111111111111</v>
+        <v>0.4609292929292929</v>
       </c>
       <c r="B48" t="n">
-        <v>5649.234846605662</v>
+        <v>5011.712176172477</v>
       </c>
       <c r="C48" t="n">
-        <v>397.8254013644087</v>
+        <v>273.1384655339663</v>
       </c>
       <c r="D48" t="n">
-        <v>42.44736933314307</v>
+        <v>41.12883319598829</v>
       </c>
       <c r="E48" t="n">
-        <v>0.7978095192025172</v>
+        <v>0.695979720649346</v>
       </c>
       <c r="F48" t="n">
-        <v>10.20091763212895</v>
+        <v>8.911529109449347</v>
       </c>
       <c r="G48" t="n">
-        <v>0.9444777817976872</v>
+        <v>0.4610876513283725</v>
       </c>
       <c r="H48" t="n">
-        <v>2.091880620133782e+21</v>
+        <v>4.888964875956107e+20</v>
       </c>
       <c r="I48" t="n">
-        <v>1.680123296257771e+21</v>
+        <v>3.412010158855571e+20</v>
+      </c>
+      <c r="J48" t="n">
+        <v>0.6979003215252806</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>1.133222222222222</v>
+        <v>0.4709494949494949</v>
       </c>
       <c r="B49" t="n">
-        <v>5634.26828923886</v>
+        <v>5010.552524346482</v>
       </c>
       <c r="C49" t="n">
-        <v>396.1749787538564</v>
+        <v>272.6522252333794</v>
       </c>
       <c r="D49" t="n">
-        <v>42.44932522308279</v>
+        <v>41.12834870579212</v>
       </c>
       <c r="E49" t="n">
-        <v>0.7987262542829142</v>
+        <v>0.6950623610341256</v>
       </c>
       <c r="F49" t="n">
-        <v>10.16551480456492</v>
+        <v>8.909572179082701</v>
       </c>
       <c r="G49" t="n">
-        <v>0.9337184747141217</v>
+        <v>0.459952697964524</v>
       </c>
       <c r="H49" t="n">
-        <v>2.088701915602762e+21</v>
+        <v>4.885523720166514e+20</v>
       </c>
       <c r="I49" t="n">
-        <v>1.679295998340352e+21</v>
+        <v>3.405097111677683e+20</v>
+      </c>
+      <c r="J49" t="n">
+        <v>0.6969768865561105</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>1.157333333333333</v>
+        <v>0.4809696969696969</v>
       </c>
       <c r="B50" t="n">
-        <v>5619.25411122695</v>
+        <v>5009.243408329758</v>
       </c>
       <c r="C50" t="n">
-        <v>394.4219787276704</v>
+        <v>272.4725864229097</v>
       </c>
       <c r="D50" t="n">
-        <v>42.45090663873077</v>
+        <v>41.12808221829464</v>
       </c>
       <c r="E50" t="n">
-        <v>0.7994470908308416</v>
+        <v>0.6949675177460171</v>
       </c>
       <c r="F50" t="n">
-        <v>10.13025857215438</v>
+        <v>8.907364576024039</v>
       </c>
       <c r="G50" t="n">
-        <v>0.9227767353990672</v>
+        <v>0.4592953783246904</v>
       </c>
       <c r="H50" t="n">
-        <v>2.084752093869489e+21</v>
+        <v>4.883011756002715e+20</v>
       </c>
       <c r="I50" t="n">
-        <v>1.677433101813415e+21</v>
+        <v>3.402862429415725e+20</v>
+      </c>
+      <c r="J50" t="n">
+        <v>0.696877787613877</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>1.181444444444445</v>
+        <v>0.490989898989899</v>
       </c>
       <c r="B51" t="n">
-        <v>5604.169134520881</v>
+        <v>5007.814795656563</v>
       </c>
       <c r="C51" t="n">
-        <v>392.6231385400706</v>
+        <v>272.5604633949138</v>
       </c>
       <c r="D51" t="n">
-        <v>42.45215118110797</v>
+        <v>41.12798052409231</v>
       </c>
       <c r="E51" t="n">
-        <v>0.8000910007326251</v>
+        <v>0.6955883568912283</v>
       </c>
       <c r="F51" t="n">
-        <v>10.09509676029493</v>
+        <v>8.904957421405568</v>
       </c>
       <c r="G51" t="n">
-        <v>0.9117780405252199</v>
+        <v>0.4590570126468261</v>
       </c>
       <c r="H51" t="n">
-        <v>2.080103150576466e+21</v>
+        <v>4.881195740780328e+20</v>
       </c>
       <c r="I51" t="n">
-        <v>1.674842317082653e+21</v>
+        <v>3.404614397660494e+20</v>
+      </c>
+      <c r="J51" t="n">
+        <v>0.6974959781301904</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>1.205555555555555</v>
+        <v>0.501010101010101</v>
       </c>
       <c r="B52" t="n">
-        <v>5588.989419284783</v>
+        <v>5006.295202613666</v>
       </c>
       <c r="C52" t="n">
-        <v>390.8420867102699</v>
+        <v>272.8731822896593</v>
       </c>
       <c r="D52" t="n">
-        <v>42.45309874446689</v>
+        <v>41.12799288284069</v>
       </c>
       <c r="E52" t="n">
-        <v>0.8007938172330691</v>
+        <v>0.6968092531188553</v>
       </c>
       <c r="F52" t="n">
-        <v>10.05997700811728</v>
+        <v>8.902399237515429</v>
       </c>
       <c r="G52" t="n">
-        <v>0.9008608907881854</v>
+        <v>0.4591722559551613</v>
       </c>
       <c r="H52" t="n">
-        <v>2.074831799610177e+21</v>
+        <v>4.879853797073364e+20</v>
       </c>
       <c r="I52" t="n">
-        <v>1.671868721536028e+21</v>
+        <v>3.409629923283725e+20</v>
+      </c>
+      <c r="J52" t="n">
+        <v>0.6987155896614383</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>1.229666666666667</v>
+        <v>0.5110303030303029</v>
       </c>
       <c r="B53" t="n">
-        <v>5573.690176140897</v>
+        <v>5004.703977094577</v>
       </c>
       <c r="C53" t="n">
-        <v>389.1502835379565</v>
+        <v>273.3500279735092</v>
       </c>
       <c r="D53" t="n">
-        <v>42.45379180289851</v>
+        <v>41.12808465902532</v>
       </c>
       <c r="E53" t="n">
-        <v>0.8017106746159619</v>
+        <v>0.6984708670485992</v>
       </c>
       <c r="F53" t="n">
-        <v>10.02484691608355</v>
+        <v>8.899722888297129</v>
       </c>
       <c r="G53" t="n">
-        <v>0.8901800286235063</v>
+        <v>0.4595432177433801</v>
       </c>
       <c r="H53" t="n">
-        <v>2.069019807258406e+21</v>
+        <v>4.878834495419715e+20</v>
       </c>
       <c r="I53" t="n">
-        <v>1.668898846735791e+21</v>
+        <v>3.417022955887359e+20</v>
+      </c>
+      <c r="J53" t="n">
+        <v>0.7003768951570882</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>1.253777777777778</v>
+        <v>0.521050505050505</v>
       </c>
       <c r="B54" t="n">
-        <v>5558.245661700905</v>
+        <v>5003.068310842026</v>
       </c>
       <c r="C54" t="n">
-        <v>387.6280823666199</v>
+        <v>273.9433216102037</v>
       </c>
       <c r="D54" t="n">
-        <v>42.45427574133755</v>
+        <v>41.12820724761006</v>
       </c>
       <c r="E54" t="n">
-        <v>0.8030188135523921</v>
+        <v>0.7004446377763527</v>
       </c>
       <c r="F54" t="n">
-        <v>9.989653130985156</v>
+        <v>8.89697433748217</v>
       </c>
       <c r="G54" t="n">
-        <v>0.8799002253893626</v>
+        <v>0.4600964915639088</v>
       </c>
       <c r="H54" t="n">
-        <v>2.062754195797825e+21</v>
+        <v>4.877925679238285e+20</v>
       </c>
       <c r="I54" t="n">
-        <v>1.666365186744255e+21</v>
+        <v>3.426016263931825e+20</v>
+      </c>
+      <c r="J54" t="n">
+        <v>0.7023510584660685</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>1.277888888888889</v>
+        <v>0.531070707070707</v>
       </c>
       <c r="B55" t="n">
-        <v>5542.629050179999</v>
+        <v>5001.417515137704</v>
       </c>
       <c r="C55" t="n">
-        <v>386.3659273690894</v>
+        <v>274.6077124938547</v>
       </c>
       <c r="D55" t="n">
-        <v>42.45459924448167</v>
+        <v>41.12830815751018</v>
       </c>
       <c r="E55" t="n">
-        <v>0.8049208102583462</v>
+        <v>0.702606999523858</v>
       </c>
       <c r="F55" t="n">
-        <v>9.954342134330481</v>
+        <v>8.894203213798219</v>
       </c>
       <c r="G55" t="n">
-        <v>0.8702074680494088</v>
+        <v>0.4607629784668841</v>
       </c>
       <c r="H55" t="n">
-        <v>2.056127917164597e+21</v>
+        <v>4.876898463507184e+20</v>
       </c>
       <c r="I55" t="n">
-        <v>1.664752380283152e+21</v>
+        <v>3.435844501940445e+20</v>
+      </c>
+      <c r="J55" t="n">
+        <v>0.7045142579141547</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>1.302</v>
+        <v>0.5410909090909091</v>
       </c>
       <c r="B56" t="n">
-        <v>5526.812271232116</v>
+        <v>4999.781414375433</v>
       </c>
       <c r="C56" t="n">
-        <v>385.4657054816606</v>
+        <v>275.2970837344969</v>
       </c>
       <c r="D56" t="n">
-        <v>42.45481476178449</v>
+        <v>41.12833383976175</v>
       </c>
       <c r="E56" t="n">
-        <v>0.8076482974467386</v>
+        <v>0.7048318782305152</v>
       </c>
       <c r="F56" t="n">
-        <v>9.918859286347399</v>
+        <v>8.891459298148982</v>
       </c>
       <c r="G56" t="n">
-        <v>0.8613042763358213</v>
+        <v>0.4614736165426063</v>
       </c>
       <c r="H56" t="n">
-        <v>2.049240325371058e+21</v>
+        <v>4.875519123445695e+20</v>
       </c>
       <c r="I56" t="n">
-        <v>1.664603973281986e+21</v>
+        <v>3.445725210640738e+20</v>
+      </c>
+      <c r="J56" t="n">
+        <v>0.7067401692818153</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>1.326111111111111</v>
+        <v>0.5511111111111111</v>
       </c>
       <c r="B57" t="n">
-        <v>5510.765800557646</v>
+        <v>4998.19037629182</v>
       </c>
       <c r="C57" t="n">
-        <v>385.0422721643881</v>
+        <v>275.9645107383425</v>
       </c>
       <c r="D57" t="n">
-        <v>42.45497907297716</v>
+        <v>41.12822963017935</v>
       </c>
       <c r="E57" t="n">
-        <v>0.81146625692882</v>
+        <v>0.7069905519603342</v>
       </c>
       <c r="F57" t="n">
-        <v>9.883149024166009</v>
+        <v>8.888793526240681</v>
       </c>
       <c r="G57" t="n">
-        <v>0.8534143256203002</v>
+        <v>0.4621576205701751</v>
       </c>
       <c r="H57" t="n">
-        <v>2.042198099253968e+21</v>
+        <v>4.873549484153519e+20</v>
       </c>
       <c r="I57" t="n">
-        <v>1.6665311081057e+21</v>
+        <v>3.454858310766766e+20</v>
+      </c>
+      <c r="J57" t="n">
+        <v>0.7088998115234764</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>1.350222222222222</v>
+        <v>0.5611313131313131</v>
       </c>
       <c r="B58" t="n">
-        <v>5494.589457437525</v>
+        <v>4996.675327695641</v>
       </c>
       <c r="C58" t="n">
-        <v>385.0178853659327</v>
+        <v>276.5622378586656</v>
       </c>
       <c r="D58" t="n">
-        <v>42.45496172295099</v>
+        <v>41.12793972402097</v>
       </c>
       <c r="E58" t="n">
-        <v>0.8161995862582315</v>
+        <v>0.7089515915868161</v>
       </c>
       <c r="F58" t="n">
-        <v>9.847442144928626</v>
+        <v>8.886257442793328</v>
       </c>
       <c r="G58" t="n">
-        <v>0.8463854000918687</v>
+        <v>0.4627439569664679</v>
       </c>
       <c r="H58" t="n">
-        <v>2.03478452751195e+21</v>
+        <v>4.870746735639404e+20</v>
       </c>
       <c r="I58" t="n">
-        <v>1.669973245461257e+21</v>
+        <v>3.462426330869277e+20</v>
+      </c>
+      <c r="J58" t="n">
+        <v>0.7108615000518498</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>1.374333333333333</v>
+        <v>0.5711515151515151</v>
       </c>
       <c r="B59" t="n">
-        <v>5478.715121117533</v>
+        <v>4995.267754655826</v>
       </c>
       <c r="C59" t="n">
-        <v>385.0954760663198</v>
+        <v>277.0416745095049</v>
       </c>
       <c r="D59" t="n">
-        <v>42.45414047649223</v>
+        <v>41.12740718508485</v>
       </c>
       <c r="E59" t="n">
-        <v>0.8211016824459619</v>
+        <v>0.7105808878292444</v>
       </c>
       <c r="F59" t="n">
-        <v>9.812686233898372</v>
+        <v>8.883903260691463</v>
       </c>
       <c r="G59" t="n">
-        <v>0.8397342446788573</v>
+        <v>0.4631603978721473</v>
       </c>
       <c r="H59" t="n">
-        <v>2.02593840881972e+21</v>
+        <v>4.866863873602717e+20</v>
       </c>
       <c r="I59" t="n">
-        <v>1.67251159887966e+21</v>
+        <v>3.467596055856158e+20</v>
+      </c>
+      <c r="J59" t="n">
+        <v>0.7124908659689418</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>1.398444444444444</v>
+        <v>0.5811717171717171</v>
       </c>
       <c r="B60" t="n">
-        <v>5463.186422167993</v>
+        <v>4993.999686072772</v>
       </c>
       <c r="C60" t="n">
-        <v>385.3774099477336</v>
+        <v>277.3534120820845</v>
       </c>
       <c r="D60" t="n">
-        <v>42.45245622310724</v>
+        <v>41.12657399173558</v>
       </c>
       <c r="E60" t="n">
-        <v>0.8263807192073291</v>
+        <v>0.7117417709039385</v>
       </c>
       <c r="F60" t="n">
-        <v>9.778958686306533</v>
+        <v>8.881783991723006</v>
       </c>
       <c r="G60" t="n">
-        <v>0.8336940169870687</v>
+        <v>0.4633337658564485</v>
       </c>
       <c r="H60" t="n">
-        <v>2.015577377387194e+21</v>
+        <v>4.861650492808792e+20</v>
       </c>
       <c r="I60" t="n">
-        <v>1.674474572022483e+21</v>
+        <v>3.469521626823967e+20</v>
+      </c>
+      <c r="J60" t="n">
+        <v>0.7136509775756154</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>1.422555555555556</v>
+        <v>0.5911919191919192</v>
       </c>
       <c r="B61" t="n">
-        <v>5447.936250308257</v>
+        <v>4992.903659578667</v>
       </c>
       <c r="C61" t="n">
-        <v>385.8407722336025</v>
+        <v>277.4472629831865</v>
       </c>
       <c r="D61" t="n">
-        <v>42.45001567805873</v>
+        <v>41.12538112229571</v>
       </c>
       <c r="E61" t="n">
-        <v>0.832012875486343</v>
+        <v>0.7122952288931591</v>
       </c>
       <c r="F61" t="n">
-        <v>9.746096603305249</v>
+        <v>8.879953657996625</v>
       </c>
       <c r="G61" t="n">
-        <v>0.8281753829735223</v>
+        <v>0.4631898176242984</v>
       </c>
       <c r="H61" t="n">
-        <v>2.00390745263535e+21</v>
+        <v>4.854853954818129e+20</v>
       </c>
       <c r="I61" t="n">
-        <v>1.67594986902708e+21</v>
+        <v>3.46734911048088e+20</v>
+      </c>
+      <c r="J61" t="n">
+        <v>0.7142025574301282</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>1.446666666666667</v>
+        <v>0.6012121212121212</v>
       </c>
       <c r="B62" t="n">
-        <v>5432.888930005381</v>
+        <v>4992.012668798346</v>
       </c>
       <c r="C62" t="n">
-        <v>386.4592656016461</v>
+        <v>277.2723230252659</v>
       </c>
       <c r="D62" t="n">
-        <v>42.44694289912599</v>
+        <v>41.12376868202136</v>
       </c>
       <c r="E62" t="n">
-        <v>0.8379691578673398</v>
+        <v>0.7121002303951374</v>
       </c>
       <c r="F62" t="n">
-        <v>9.713923899885557</v>
+        <v>8.878466531123923</v>
       </c>
       <c r="G62" t="n">
-        <v>0.8230803817083117</v>
+        <v>0.4626535546111911</v>
       </c>
       <c r="H62" t="n">
-        <v>1.991164563306649e+21</v>
+        <v>4.846220367576347e+20</v>
       </c>
       <c r="I62" t="n">
-        <v>1.677042705422484e+21</v>
+        <v>3.460222217329569e+20</v>
+      </c>
+      <c r="J62" t="n">
+        <v>0.7140043074558056</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>1.470777777777778</v>
+        <v>0.6112323232323232</v>
       </c>
       <c r="B63" t="n">
-        <v>5417.959152873505</v>
+        <v>4991.355906906737</v>
       </c>
       <c r="C63" t="n">
-        <v>387.2028318546397</v>
+        <v>276.7838467100828</v>
       </c>
       <c r="D63" t="n">
-        <v>42.44338149825234</v>
+        <v>41.12168351098945</v>
       </c>
       <c r="E63" t="n">
-        <v>0.8442149426207503</v>
+        <v>0.7110327871326356</v>
       </c>
       <c r="F63" t="n">
-        <v>9.682249193740315</v>
+        <v>8.877370985904804</v>
       </c>
       <c r="G63" t="n">
-        <v>0.818300954950596</v>
+        <v>0.4616588869306208</v>
       </c>
       <c r="H63" t="n">
-        <v>1.977616226872728e+21</v>
+        <v>4.835528950903057e+20</v>
       </c>
       <c r="I63" t="n">
-        <v>1.677878595287862e+21</v>
+        <v>3.447403342233217e+20</v>
+      </c>
+      <c r="J63" t="n">
+        <v>0.7129320033518565</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>1.494888888888889</v>
+        <v>0.6212525252525252</v>
       </c>
       <c r="B64" t="n">
-        <v>5403.057857112466</v>
+        <v>4990.924163798168</v>
       </c>
       <c r="C64" t="n">
-        <v>388.0382444678225</v>
+        <v>275.9990747686032</v>
       </c>
       <c r="D64" t="n">
-        <v>42.43947974780703</v>
+        <v>41.11914094418537</v>
       </c>
       <c r="E64" t="n">
-        <v>0.8507094514722549</v>
+        <v>0.709139451868979</v>
       </c>
       <c r="F64" t="n">
-        <v>9.65087918546697</v>
+        <v>8.876650877847107</v>
       </c>
       <c r="G64" t="n">
-        <v>0.8137235145428257</v>
+        <v>0.4602322140070574</v>
       </c>
       <c r="H64" t="n">
-        <v>1.96353266816414e+21</v>
+        <v>4.822858663422413e+20</v>
       </c>
       <c r="I64" t="n">
-        <v>1.67858014936189e+21</v>
+        <v>3.429208269317797e+20</v>
+      </c>
+      <c r="J64" t="n">
+        <v>0.711032296120482</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>1.519</v>
+        <v>0.6312727272727272</v>
       </c>
       <c r="B65" t="n">
-        <v>5388.111163292194</v>
+        <v>4990.674989265088</v>
       </c>
       <c r="C65" t="n">
-        <v>388.9315828078774</v>
+        <v>274.9669041832155</v>
       </c>
       <c r="D65" t="n">
-        <v>42.43534279339602</v>
+        <v>41.11622975922878</v>
       </c>
       <c r="E65" t="n">
-        <v>0.8574051339527482</v>
+        <v>0.7065579885815213</v>
       </c>
       <c r="F65" t="n">
-        <v>9.619657901260876</v>
+        <v>8.876235480228882</v>
       </c>
       <c r="G65" t="n">
-        <v>0.8092415180419987</v>
+        <v>0.458443397190749</v>
       </c>
       <c r="H65" t="n">
-        <v>1.949100457994085e+21</v>
+        <v>4.80861380927541e+20</v>
       </c>
       <c r="I65" t="n">
-        <v>1.679193161689222e+21</v>
+        <v>3.406629690976344e+20</v>
+      </c>
+      <c r="J65" t="n">
+        <v>0.7084431867673057</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>1.543111111111111</v>
+        <v>0.6412929292929292</v>
       </c>
       <c r="B66" t="n">
-        <v>5373.040208919321</v>
+        <v>4990.570572261617</v>
       </c>
       <c r="C66" t="n">
-        <v>389.8450994803558</v>
+        <v>273.7378326358601</v>
       </c>
       <c r="D66" t="n">
-        <v>42.43108048166805</v>
+        <v>41.1130247964017</v>
       </c>
       <c r="E66" t="n">
-        <v>0.8642469609388367</v>
+        <v>0.7034291873579107</v>
       </c>
       <c r="F66" t="n">
-        <v>9.588423858768259</v>
+        <v>8.87606140716448</v>
       </c>
       <c r="G66" t="n">
-        <v>0.8047413516185148</v>
+        <v>0.4563659804827391</v>
       </c>
       <c r="H66" t="n">
-        <v>1.934508851569727e+21</v>
+        <v>4.793133050302642e+20</v>
       </c>
       <c r="I66" t="n">
-        <v>1.679758432215116e+21</v>
+        <v>3.380624168054349e+20</v>
+      </c>
+      <c r="J66" t="n">
+        <v>0.7053057222855297</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>1.567222222222222</v>
+        <v>0.6513131313131313</v>
       </c>
       <c r="B67" t="n">
-        <v>5357.754590491518</v>
+        <v>4990.581111428913</v>
       </c>
       <c r="C67" t="n">
-        <v>390.7359371386785</v>
+        <v>272.3641640912656</v>
       </c>
       <c r="D67" t="n">
-        <v>42.42682259469594</v>
+        <v>41.10957748792394</v>
       </c>
       <c r="E67" t="n">
-        <v>0.8711715521359316</v>
+        <v>0.6998962897046821</v>
       </c>
       <c r="F67" t="n">
-        <v>9.556997365517248</v>
+        <v>8.876078976957585</v>
       </c>
       <c r="G67" t="n">
-        <v>0.8000960980116465</v>
+        <v>0.4540786837430408</v>
       </c>
       <c r="H67" t="n">
-        <v>1.919975941759791e+21</v>
+        <v>4.776647545202592e+20</v>
       </c>
       <c r="I67" t="n">
-        <v>1.680333982233856e+21</v>
+        <v>3.352076572799939e+20</v>
+      </c>
+      <c r="J67" t="n">
+        <v>0.7017634315863612</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>1.591333333333333</v>
+        <v>0.6613333333333333</v>
       </c>
       <c r="B68" t="n">
-        <v>5342.150768603615</v>
+        <v>4990.765304193316</v>
       </c>
       <c r="C68" t="n">
-        <v>391.5554794908172</v>
+        <v>271.0622854620765</v>
       </c>
       <c r="D68" t="n">
-        <v>42.42272192636074</v>
+        <v>41.10578185915936</v>
       </c>
       <c r="E68" t="n">
-        <v>0.8781060865275266</v>
+        <v>0.6964994283053039</v>
       </c>
       <c r="F68" t="n">
-        <v>9.525177710609224</v>
+        <v>8.876386043794158</v>
       </c>
       <c r="G68" t="n">
-        <v>0.7951652899275156</v>
+        <v>0.4519575280531566</v>
       </c>
       <c r="H68" t="n">
-        <v>1.905752551615774e+21</v>
+        <v>4.758716150479112e+20</v>
       </c>
       <c r="I68" t="n">
-        <v>1.680998279009772e+21</v>
+        <v>3.323287773008191e+20</v>
+      </c>
+      <c r="J68" t="n">
+        <v>0.6983580587536408</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>1.615444444444444</v>
+        <v>0.6713535353535353</v>
       </c>
       <c r="B69" t="n">
-        <v>5326.187216900278</v>
+        <v>4991.153973726557</v>
       </c>
       <c r="C69" t="n">
-        <v>392.1298260208633</v>
+        <v>269.9983334745859</v>
       </c>
       <c r="D69" t="n">
-        <v>42.41883774574287</v>
+        <v>41.10158156725019</v>
       </c>
       <c r="E69" t="n">
-        <v>0.8846734294836756</v>
+        <v>0.6936575393231553</v>
       </c>
       <c r="F69" t="n">
-        <v>9.492896580298158</v>
+        <v>8.877034144801742</v>
       </c>
       <c r="G69" t="n">
-        <v>0.7895851457924128</v>
+        <v>0.450287189698961</v>
       </c>
       <c r="H69" t="n">
-        <v>1.891931003706579e+21</v>
+        <v>4.739116069389348e+20</v>
       </c>
       <c r="I69" t="n">
-        <v>1.681122445692927e+21</v>
+        <v>3.296101401782611e+20</v>
+      </c>
+      <c r="J69" t="n">
+        <v>0.6955097434883727</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>1.639555555555555</v>
+        <v>0.6813737373737373</v>
       </c>
       <c r="B70" t="n">
-        <v>5310.004118142854</v>
+        <v>4991.690653567344</v>
       </c>
       <c r="C70" t="n">
-        <v>392.2377210927443</v>
+        <v>269.179026872908</v>
       </c>
       <c r="D70" t="n">
-        <v>42.41494501355352</v>
+        <v>41.09707556292945</v>
       </c>
       <c r="E70" t="n">
-        <v>0.890318923177789</v>
+        <v>0.691403948026175</v>
       </c>
       <c r="F70" t="n">
-        <v>9.460451193852327</v>
+        <v>8.877929370783923</v>
       </c>
       <c r="G70" t="n">
-        <v>0.7829874549126753</v>
+        <v>0.4490635281959622</v>
       </c>
       <c r="H70" t="n">
-        <v>1.878139307529443e+21</v>
+        <v>4.71828541033044e+20</v>
       </c>
       <c r="I70" t="n">
-        <v>1.679352428335693e+21</v>
+        <v>3.27095951693394e+20</v>
+      </c>
+      <c r="J70" t="n">
+        <v>0.6932517286411595</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>1.663666666666667</v>
+        <v>0.6913939393939393</v>
       </c>
       <c r="B71" t="n">
-        <v>5293.63429164332</v>
+        <v>4992.318088047396</v>
       </c>
       <c r="C71" t="n">
-        <v>391.9250346812698</v>
+        <v>268.6108955289205</v>
       </c>
       <c r="D71" t="n">
-        <v>42.41098241005045</v>
+        <v>41.09236414905071</v>
       </c>
       <c r="E71" t="n">
-        <v>0.8951196653206825</v>
+        <v>0.6897712519082061</v>
       </c>
       <c r="F71" t="n">
-        <v>9.427917148536642</v>
+        <v>8.878976297535356</v>
       </c>
       <c r="G71" t="n">
-        <v>0.7755019118342886</v>
+        <v>0.4482822872566481</v>
       </c>
       <c r="H71" t="n">
-        <v>1.864278422838299e+21</v>
+        <v>4.696661686604013e+20</v>
       </c>
       <c r="I71" t="n">
-        <v>1.675783324150544e+21</v>
+        <v>3.248288856858247e+20</v>
+      </c>
+      <c r="J71" t="n">
+        <v>0.6916165296987715</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>1.687777777777778</v>
+        <v>0.7014141414141414</v>
       </c>
       <c r="B72" t="n">
-        <v>5277.080412799361</v>
+        <v>4992.978240537172</v>
       </c>
       <c r="C72" t="n">
-        <v>391.2007322545457</v>
+        <v>268.3003725794496</v>
       </c>
       <c r="D72" t="n">
-        <v>42.40693455505438</v>
+        <v>41.08754891501368</v>
       </c>
       <c r="E72" t="n">
-        <v>0.8990797121261545</v>
+        <v>0.6887916789282157</v>
       </c>
       <c r="F72" t="n">
-        <v>9.395307969590487</v>
+        <v>8.880078138911619</v>
       </c>
       <c r="G72" t="n">
-        <v>0.7671700557077884</v>
+        <v>0.4479391406115175</v>
       </c>
       <c r="H72" t="n">
-        <v>1.850325248891415e+21</v>
+        <v>4.674680558661e+20</v>
       </c>
       <c r="I72" t="n">
-        <v>1.670436703047581e+21</v>
+        <v>3.228504050101221e+20</v>
+      </c>
+      <c r="J72" t="n">
+        <v>0.6906362925953561</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>1.711888888888889</v>
+        <v>0.7114343434343434</v>
       </c>
       <c r="B73" t="n">
-        <v>5260.346214588201</v>
+        <v>4993.612276065678</v>
       </c>
       <c r="C73" t="n">
-        <v>390.0775665700497</v>
+        <v>268.2538972350293</v>
       </c>
       <c r="D73" t="n">
-        <v>42.40278345251333</v>
+        <v>41.08273273965982</v>
       </c>
       <c r="E73" t="n">
-        <v>0.902211337801164</v>
+        <v>0.6884974961107307</v>
       </c>
       <c r="F73" t="n">
-        <v>9.362639856704375</v>
+        <v>8.88113699415397</v>
       </c>
       <c r="G73" t="n">
-        <v>0.7580416909894105</v>
+        <v>0.4480297566782442</v>
       </c>
       <c r="H73" t="n">
-        <v>1.836253226317432e+21</v>
+        <v>4.652775334337456e+20</v>
       </c>
       <c r="I73" t="n">
-        <v>1.663345993999817e+21</v>
+        <v>3.212011822269836e+20</v>
+      </c>
+      <c r="J73" t="n">
+        <v>0.6903432019520063</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>1.736</v>
+        <v>0.7214545454545453</v>
       </c>
       <c r="B74" t="n">
-        <v>5243.43671445742</v>
+        <v>4994.16051697029</v>
       </c>
       <c r="C74" t="n">
-        <v>388.5728173449978</v>
+        <v>268.4780283691682</v>
       </c>
       <c r="D74" t="n">
-        <v>42.3985079931317</v>
+        <v>41.07801986603815</v>
       </c>
       <c r="E74" t="n">
-        <v>0.9045369614352856</v>
+        <v>0.6889214690779238</v>
       </c>
       <c r="F74" t="n">
-        <v>9.329930635618192</v>
+        <v>8.882052747722685</v>
       </c>
       <c r="G74" t="n">
-        <v>0.748174537995298</v>
+        <v>0.4485496654359607</v>
       </c>
       <c r="H74" t="n">
-        <v>1.822031413154361e+21</v>
+        <v>4.631376485107426e+20</v>
       </c>
       <c r="I74" t="n">
-        <v>1.654558704278086e+21</v>
+        <v>3.199215652698417e+20</v>
+      </c>
+      <c r="J74" t="n">
+        <v>0.6907699391284124</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>1.760111111111111</v>
+        <v>0.7314747474747474</v>
       </c>
       <c r="B75" t="n">
-        <v>5226.358486022068</v>
+        <v>4994.562370102115</v>
       </c>
       <c r="C75" t="n">
-        <v>386.7091653590472</v>
+        <v>268.9795693560213</v>
       </c>
       <c r="D75" t="n">
-        <v>42.39408335897691</v>
+        <v>41.07351605172392</v>
       </c>
       <c r="E75" t="n">
-        <v>0.9060914602747515</v>
+        <v>0.6900973747559159</v>
       </c>
       <c r="F75" t="n">
-        <v>9.297201047746931</v>
+        <v>8.882724263996769</v>
       </c>
       <c r="G75" t="n">
-        <v>0.7376364836776851</v>
+        <v>0.4494944976472375</v>
       </c>
       <c r="H75" t="n">
-        <v>1.807623894791161e+21</v>
+        <v>4.610913103028952e+20</v>
       </c>
       <c r="I75" t="n">
-        <v>1.644139525503315e+21</v>
+        <v>3.190522223101972e+20</v>
+      </c>
+      <c r="J75" t="n">
+        <v>0.6919501955059807</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>1.784222222222222</v>
+        <v>0.7414949494949494</v>
       </c>
       <c r="B76" t="n">
-        <v>5209.119983727565</v>
+        <v>4994.756223882555</v>
       </c>
       <c r="C76" t="n">
-        <v>384.5157253925485</v>
+        <v>269.7657050492285</v>
       </c>
       <c r="D76" t="n">
-        <v>42.38948031137851</v>
+        <v>41.06932879895636</v>
       </c>
       <c r="E76" t="n">
-        <v>0.9069249442056474</v>
+        <v>0.6920605715132587</v>
       </c>
       <c r="F76" t="n">
-        <v>9.264474838848272</v>
+        <v>8.883048203162719</v>
       </c>
       <c r="G76" t="n">
-        <v>0.7265070657603346</v>
+        <v>0.4508599368658304</v>
       </c>
       <c r="H76" t="n">
-        <v>1.792988809801369e+21</v>
+        <v>4.591813860002281e+20</v>
       </c>
       <c r="I76" t="n">
-        <v>1.63217370706996e+21</v>
+        <v>3.186347992084401e+20</v>
+      </c>
+      <c r="J76" t="n">
+        <v>0.6939192417705753</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>1.808333333333333</v>
+        <v>0.7515151515151515</v>
       </c>
       <c r="B77" t="n">
-        <v>5191.731929780948</v>
+        <v>4994.681559744614</v>
       </c>
       <c r="C77" t="n">
-        <v>382.0292666727734</v>
+        <v>270.8405019681866</v>
       </c>
       <c r="D77" t="n">
-        <v>42.38466434048384</v>
+        <v>41.06556368180387</v>
       </c>
       <c r="E77" t="n">
-        <v>0.9071060798356454</v>
+        <v>0.6948386434413233</v>
       </c>
       <c r="F77" t="n">
-        <v>9.231779598918399</v>
+        <v>8.882923435729678</v>
       </c>
       <c r="G77" t="n">
-        <v>0.7148784941978448</v>
+        <v>0.4526362473746221</v>
       </c>
       <c r="H77" t="n">
-        <v>1.778077354603917e+21</v>
+        <v>4.574493396842419e+20</v>
       </c>
       <c r="I77" t="n">
-        <v>1.618771117188415e+21</v>
+        <v>3.187070368213508e+20</v>
+      </c>
+      <c r="J77" t="n">
+        <v>0.6967045510249089</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>1.832444444444445</v>
+        <v>0.7615353535353535</v>
       </c>
       <c r="B78" t="n">
-        <v>5174.207773770594</v>
+        <v>4994.313515745921</v>
       </c>
       <c r="C78" t="n">
-        <v>379.2956543723788</v>
+        <v>272.1486631435228</v>
       </c>
       <c r="D78" t="n">
-        <v>42.37959465177911</v>
+        <v>41.06226308353234</v>
       </c>
       <c r="E78" t="n">
-        <v>0.9067260679748627</v>
+        <v>0.6982976254416819</v>
       </c>
       <c r="F78" t="n">
-        <v>9.199146847634337</v>
+        <v>8.882308416173705</v>
       </c>
       <c r="G78" t="n">
-        <v>0.7028583098377822</v>
+        <v>0.4547234221485024</v>
       </c>
       <c r="H78" t="n">
-        <v>1.76283245327639e+21</v>
+        <v>4.559104044863381e+20</v>
       </c>
       <c r="I78" t="n">
-        <v>1.604070833748689e+21</v>
+        <v>3.192155691296596e+20</v>
+      </c>
+      <c r="J78" t="n">
+        <v>0.7001717135394423</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>1.856555555555556</v>
+        <v>0.7715555555555556</v>
       </c>
       <c r="B79" t="n">
-        <v>5156.471799211699</v>
+        <v>4993.653072337557</v>
       </c>
       <c r="C79" t="n">
-        <v>376.3580862322991</v>
+        <v>273.5914311770517</v>
       </c>
       <c r="D79" t="n">
-        <v>42.37447276217766</v>
+        <v>41.05942366121418</v>
       </c>
       <c r="E79" t="n">
-        <v>0.9059034645210817</v>
+        <v>0.7021852785781432</v>
       </c>
       <c r="F79" t="n">
-        <v>9.166443817660067</v>
+        <v>8.881205126334988</v>
       </c>
       <c r="G79" t="n">
-        <v>0.6905113921650451</v>
+        <v>0.4569553873637509</v>
       </c>
       <c r="H79" t="n">
-        <v>1.747591638275682e+21</v>
+        <v>4.545612494141262e+20</v>
       </c>
       <c r="I79" t="n">
-        <v>1.588613426195048e+21</v>
+        <v>3.200419396053228e+20</v>
+      </c>
+      <c r="J79" t="n">
+        <v>0.7040678016830905</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>1.880666666666667</v>
+        <v>0.7815757575757575</v>
       </c>
       <c r="B80" t="n">
-        <v>5137.976748897547</v>
+        <v>4992.701596016118</v>
       </c>
       <c r="C80" t="n">
-        <v>373.2228339663386</v>
+        <v>275.0678329626344</v>
       </c>
       <c r="D80" t="n">
-        <v>42.37078084555837</v>
+        <v>41.05704153294018</v>
       </c>
       <c r="E80" t="n">
-        <v>0.9048360599738531</v>
+        <v>0.7062436388460774</v>
       </c>
       <c r="F80" t="n">
-        <v>9.132686686831338</v>
+        <v>8.879616399564217</v>
       </c>
       <c r="G80" t="n">
-        <v>0.677653089429313</v>
+        <v>0.4591624891384374</v>
       </c>
       <c r="H80" t="n">
-        <v>1.734739457221081e+21</v>
+        <v>4.533985935465079e+20</v>
       </c>
       <c r="I80" t="n">
-        <v>1.574923762067214e+21</v>
+        <v>3.210670271047199e+20</v>
+      </c>
+      <c r="J80" t="n">
+        <v>0.7081341487923827</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>1.904777777777778</v>
+        <v>0.7915959595959595</v>
       </c>
       <c r="B81" t="n">
-        <v>5118.695649222355</v>
+        <v>4991.460453945701</v>
       </c>
       <c r="C81" t="n">
-        <v>370.0141920975998</v>
+        <v>276.4750995565878</v>
       </c>
       <c r="D81" t="n">
-        <v>42.36868078806754</v>
+        <v>41.05511295814121</v>
       </c>
       <c r="E81" t="n">
-        <v>0.9038278711059416</v>
+        <v>0.7102098916044546</v>
       </c>
       <c r="F81" t="n">
-        <v>9.097869082395464</v>
+        <v>8.877545378938654</v>
       </c>
       <c r="G81" t="n">
-        <v>0.6645179620535203</v>
+        <v>0.4611724729585946</v>
       </c>
       <c r="H81" t="n">
-        <v>1.724500552378725e+21</v>
+        <v>4.524194792664387e+20</v>
       </c>
       <c r="I81" t="n">
-        <v>1.563732957395926e+21</v>
+        <v>3.221711816218903e+20</v>
+      </c>
+      <c r="J81" t="n">
+        <v>0.7121072287697792</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>1.928888888888889</v>
+        <v>0.8016161616161616</v>
       </c>
       <c r="B82" t="n">
-        <v>5098.867770205413</v>
+        <v>4989.931023530973</v>
       </c>
       <c r="C82" t="n">
-        <v>367.0432499384945</v>
+        <v>277.7083700107743</v>
       </c>
       <c r="D82" t="n">
-        <v>42.36778611130751</v>
+        <v>41.05363431691949</v>
       </c>
       <c r="E82" t="n">
-        <v>0.9035573137855918</v>
+        <v>0.7138152920891228</v>
       </c>
       <c r="F82" t="n">
-        <v>9.062460180024248</v>
+        <v>8.87499528682212</v>
       </c>
       <c r="G82" t="n">
-        <v>0.6517640534947093</v>
+        <v>0.4628101312673722</v>
       </c>
       <c r="H82" t="n">
-        <v>1.716252618584263e+21</v>
+        <v>4.516212411591382e+20</v>
       </c>
       <c r="I82" t="n">
-        <v>1.555637141115261e+21</v>
+        <v>3.232332599386475e+20</v>
+      </c>
+      <c r="J82" t="n">
+        <v>0.7157175758806914</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>1.953</v>
+        <v>0.8116363636363636</v>
       </c>
       <c r="B83" t="n">
-        <v>5078.598091020253</v>
+        <v>4988.128812457981</v>
       </c>
       <c r="C83" t="n">
-        <v>364.3343514683032</v>
+        <v>278.6864518460231</v>
       </c>
       <c r="D83" t="n">
-        <v>42.36792636300844</v>
+        <v>41.05257696430156</v>
       </c>
       <c r="E83" t="n">
-        <v>0.9040623715761255</v>
+        <v>0.7168470445634095</v>
       </c>
       <c r="F83" t="n">
-        <v>9.026675583224097</v>
+        <v>8.871993470200033</v>
       </c>
       <c r="G83" t="n">
-        <v>0.6394650690531076</v>
+        <v>0.4639441631489672</v>
       </c>
       <c r="H83" t="n">
-        <v>1.709715489895031e+21</v>
+        <v>4.509913788276124e+20</v>
       </c>
       <c r="I83" t="n">
-        <v>1.550427585094509e+21</v>
+        <v>3.24150898269678e+20</v>
+      </c>
+      <c r="J83" t="n">
+        <v>0.7187518730675824</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>1.977111111111111</v>
+        <v>0.8216565656565656</v>
       </c>
       <c r="B84" t="n">
-        <v>5057.987300354919</v>
+        <v>4986.14075776027</v>
       </c>
       <c r="C84" t="n">
-        <v>361.8659351438147</v>
+        <v>279.457250458027</v>
       </c>
       <c r="D84" t="n">
-        <v>42.36892994202132</v>
+        <v>41.05178501815774</v>
       </c>
       <c r="E84" t="n">
-        <v>0.9052701404397201</v>
+        <v>0.7194030519981642</v>
       </c>
       <c r="F84" t="n">
-        <v>8.990714664326687</v>
+        <v>8.868685804705963</v>
       </c>
       <c r="G84" t="n">
-        <v>0.6276098672137905</v>
+        <v>0.4646789808001807</v>
       </c>
       <c r="H84" t="n">
-        <v>1.704614097139023e+21</v>
+        <v>4.504663533796993e+20</v>
       </c>
       <c r="I84" t="n">
-        <v>1.547717290897929e+21</v>
+        <v>3.24925236061886e+20</v>
+      </c>
+      <c r="J84" t="n">
+        <v>0.7213085586172638</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>2.001222222222222</v>
+        <v>0.8316767676767676</v>
       </c>
       <c r="B85" t="n">
-        <v>5037.154327736131</v>
+        <v>4984.003247430868</v>
       </c>
       <c r="C85" t="n">
-        <v>359.6074173943163</v>
+        <v>280.005730724909</v>
       </c>
       <c r="D85" t="n">
-        <v>42.37058422816678</v>
+        <v>41.05121337929859</v>
       </c>
       <c r="E85" t="n">
-        <v>0.9070768644976834</v>
+        <v>0.7214334078638226</v>
       </c>
       <c r="F85" t="n">
-        <v>8.954800496806408</v>
+        <v>8.865133767544476</v>
       </c>
       <c r="G85" t="n">
-        <v>0.6161777459100407</v>
+        <v>0.4650006734663277</v>
       </c>
       <c r="H85" t="n">
-        <v>1.700615851971829e+21</v>
+        <v>4.500286076964061e+20</v>
       </c>
       <c r="I85" t="n">
-        <v>1.547021387844194e+21</v>
+        <v>3.255226658201427e+20</v>
+      </c>
+      <c r="J85" t="n">
+        <v>0.7233377173207256</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>2.025333333333333</v>
+        <v>0.8416969696969696</v>
       </c>
       <c r="B86" t="n">
-        <v>5016.238605873115</v>
+        <v>4981.747722325322</v>
       </c>
       <c r="C86" t="n">
-        <v>357.5174413691724</v>
+        <v>280.3029866575598</v>
       </c>
       <c r="D86" t="n">
-        <v>42.3726294558368</v>
+        <v>41.05082443206364</v>
       </c>
       <c r="E86" t="n">
-        <v>0.9093411071008566</v>
+        <v>0.7228533970870922</v>
       </c>
       <c r="F86" t="n">
-        <v>8.91918038772442</v>
+        <v>8.861390655375683</v>
       </c>
       <c r="G86" t="n">
-        <v>0.6051373865172307</v>
+        <v>0.4648711175627842</v>
       </c>
       <c r="H86" t="n">
-        <v>1.697319054922226e+21</v>
+        <v>4.496636633351311e+20</v>
       </c>
       <c r="I86" t="n">
-        <v>1.547732031006883e+21</v>
+        <v>3.258957729086015e+20</v>
+      </c>
+      <c r="J86" t="n">
+        <v>0.724754520948947</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>2.049444444444445</v>
+        <v>0.8517171717171717</v>
       </c>
       <c r="B87" t="n">
-        <v>4995.402541179452</v>
+        <v>4979.424563784134</v>
       </c>
       <c r="C87" t="n">
-        <v>355.5419184336624</v>
+        <v>280.3212231232278</v>
       </c>
       <c r="D87" t="n">
-        <v>42.37475197859581</v>
+        <v>41.05052677239609</v>
       </c>
       <c r="E87" t="n">
-        <v>0.9118760168474235</v>
+        <v>0.7235751238761903</v>
       </c>
       <c r="F87" t="n">
-        <v>8.884128628746067</v>
+        <v>8.857540477644653</v>
       </c>
       <c r="G87" t="n">
-        <v>0.5944450793445841</v>
+        <v>0.4642597950149859</v>
       </c>
       <c r="H87" t="n">
-        <v>1.694240960343273e+21</v>
+        <v>4.493345206988322e+20</v>
       </c>
       <c r="I87" t="n">
-        <v>1.549091251707387e+21</v>
+        <v>3.259791712995552e+20</v>
+      </c>
+      <c r="J87" t="n">
+        <v>0.7254710160985911</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>2.073555555555556</v>
+        <v>0.8617373737373737</v>
       </c>
       <c r="B88" t="n">
-        <v>4974.834173846558</v>
+        <v>4977.085297035283</v>
       </c>
       <c r="C88" t="n">
-        <v>353.6118867579232</v>
+        <v>280.0318099900365</v>
       </c>
       <c r="D88" t="n">
-        <v>42.37657699532362</v>
+        <v>41.05022659781676</v>
       </c>
       <c r="E88" t="n">
-        <v>0.914440811701951</v>
+        <v>0.7235077091116936</v>
       </c>
       <c r="F88" t="n">
-        <v>8.849948329292992</v>
+        <v>8.853668865753043</v>
       </c>
       <c r="G88" t="n">
-        <v>0.5840439249605794</v>
+        <v>0.4631354905457295</v>
       </c>
       <c r="H88" t="n">
-        <v>1.690805566842646e+21</v>
+        <v>4.490033179335074e+20</v>
       </c>
       <c r="I88" t="n">
-        <v>1.550162792426883e+21</v>
+        <v>3.257053300556635e+20</v>
+      </c>
+      <c r="J88" t="n">
+        <v>0.7253962655658972</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>2.097666666666667</v>
+        <v>0.8717575757575757</v>
       </c>
       <c r="B89" t="n">
-        <v>4954.749986110156</v>
+        <v>4974.782606180973</v>
       </c>
       <c r="C89" t="n">
-        <v>351.6412403700655</v>
+        <v>279.4053472082883</v>
       </c>
       <c r="D89" t="n">
-        <v>42.37766088501915</v>
+        <v>41.0498276536138</v>
       </c>
       <c r="E89" t="n">
-        <v>0.9167317565013645</v>
+        <v>0.7225575808218085</v>
       </c>
       <c r="F89" t="n">
-        <v>8.816974274585844</v>
+        <v>8.849863174369188</v>
       </c>
       <c r="G89" t="n">
-        <v>0.5738614888646228</v>
+        <v>0.4614663445324418</v>
       </c>
       <c r="H89" t="n">
-        <v>1.686332596540499e+21</v>
+        <v>4.486313022443944e+20</v>
       </c>
       <c r="I89" t="n">
-        <v>1.549805988148816e+21</v>
+        <v>3.250049526125767e+20</v>
+      </c>
+      <c r="J89" t="n">
+        <v>0.7244366386978687</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>2.121777777777778</v>
+        <v>0.8817777777777778</v>
       </c>
       <c r="B90" t="n">
-        <v>4935.397786166384</v>
+        <v>4972.570326967394</v>
       </c>
       <c r="C90" t="n">
-        <v>349.5244224666977</v>
+        <v>278.4117561557844</v>
       </c>
       <c r="D90" t="n">
-        <v>42.37748340284578</v>
+        <v>41.04923123780663</v>
       </c>
       <c r="E90" t="n">
-        <v>0.9183731242764033</v>
+        <v>0.7206288826670665</v>
       </c>
       <c r="F90" t="n">
-        <v>8.785575287505598</v>
+        <v>8.846211813775959</v>
       </c>
       <c r="G90" t="n">
-        <v>0.5638081447724229</v>
+        <v>0.4592196857079004</v>
       </c>
       <c r="H90" t="n">
-        <v>1.680029031383502e+21</v>
+        <v>4.481788210207874e+20</v>
       </c>
       <c r="I90" t="n">
-        <v>1.54665587358318e+21</v>
+        <v>3.238075032345349e+20</v>
+      </c>
+      <c r="J90" t="n">
+        <v>0.7224962181323514</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>2.145888888888889</v>
+        <v>0.8917979797979797</v>
       </c>
       <c r="B91" t="n">
-        <v>4917.066672125498</v>
+        <v>4970.503415596784</v>
       </c>
       <c r="C91" t="n">
-        <v>347.12289868076</v>
+        <v>277.0203994529367</v>
       </c>
       <c r="D91" t="n">
-        <v>42.37542709131036</v>
+        <v>41.04833626997134</v>
       </c>
       <c r="E91" t="n">
-        <v>0.9188762626796562</v>
+        <v>0.7176240103774526</v>
       </c>
       <c r="F91" t="n">
-        <v>8.756168983844002</v>
+        <v>8.842804696826818</v>
       </c>
       <c r="G91" t="n">
-        <v>0.5537590990198052</v>
+        <v>0.4563621200002578</v>
       </c>
       <c r="H91" t="n">
-        <v>1.6709662238918e+21</v>
+        <v>4.476054332475996e+20</v>
       </c>
       <c r="I91" t="n">
-        <v>1.539043490652804e+21</v>
+        <v>3.220419646638197e+20</v>
+      </c>
+      <c r="J91" t="n">
+        <v>0.719477335936799</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>2.17</v>
+        <v>0.9018181818181817</v>
       </c>
       <c r="B92" t="n">
-        <v>4900.098610495746</v>
+        <v>4968.636623529658</v>
       </c>
       <c r="C92" t="n">
-        <v>344.3982686152154</v>
+        <v>275.2022892885681</v>
       </c>
       <c r="D92" t="n">
-        <v>42.37075357746467</v>
+        <v>41.04704170410221</v>
       </c>
       <c r="E92" t="n">
-        <v>0.9179885885045033</v>
+        <v>0.7134499844571233</v>
       </c>
       <c r="F92" t="n">
-        <v>8.729239272879552</v>
+        <v>8.839731055181158</v>
       </c>
       <c r="G92" t="n">
-        <v>0.5437692417649088</v>
+        <v>0.4528623371826186</v>
       </c>
       <c r="H92" t="n">
-        <v>1.658060043394954e+21</v>
+        <v>4.468709730079216e+20</v>
       </c>
       <c r="I92" t="n">
-        <v>1.525580539992009e+21</v>
+        <v>3.196409772542089e+20</v>
+      </c>
+      <c r="J92" t="n">
+        <v>0.7152869543140872</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>2.194111111111111</v>
+        <v>0.9118383838383838</v>
       </c>
       <c r="B93" t="n">
-        <v>4884.978194320148</v>
+        <v>4966.985264486981</v>
       </c>
       <c r="C93" t="n">
-        <v>341.5985999710687</v>
+        <v>272.9938295971748</v>
       </c>
       <c r="D93" t="n">
-        <v>42.36243503626753</v>
+        <v>41.04531701840001</v>
       </c>
       <c r="E93" t="n">
-        <v>0.9161715176944898</v>
+        <v>0.7081953171183651</v>
       </c>
       <c r="F93" t="n">
-        <v>8.705475630010056</v>
+        <v>8.83701487471483</v>
       </c>
       <c r="G93" t="n">
-        <v>0.5343838992291513</v>
+        <v>0.4487854883656349</v>
       </c>
       <c r="H93" t="n">
-        <v>1.639848259757582e+21</v>
+        <v>4.459638520212499e+20</v>
       </c>
       <c r="I93" t="n">
-        <v>1.505750733728418e+21</v>
+        <v>3.166405208453707e+20</v>
+      </c>
+      <c r="J93" t="n">
+        <v>0.710013870878223</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>2.218222222222222</v>
+        <v>0.9218585858585858</v>
       </c>
       <c r="B94" t="n">
-        <v>4872.150159553375</v>
+        <v>4965.534435207487</v>
       </c>
       <c r="C94" t="n">
-        <v>338.7786008097028</v>
+        <v>270.4820827351559</v>
       </c>
       <c r="D94" t="n">
-        <v>42.34945592681767</v>
+        <v>41.0431859396568</v>
       </c>
       <c r="E94" t="n">
-        <v>0.9133991505699293</v>
+        <v>0.7020894850581879</v>
       </c>
       <c r="F94" t="n">
-        <v>8.685486822642734</v>
+        <v>8.8346309457429</v>
       </c>
       <c r="G94" t="n">
-        <v>0.5258111697632626</v>
+        <v>0.444271359835794</v>
       </c>
       <c r="H94" t="n">
-        <v>1.614985283932154e+21</v>
+        <v>4.448944299706009e+20</v>
       </c>
       <c r="I94" t="n">
-        <v>1.478362667706805e+21</v>
+        <v>3.131559009305999e+20</v>
+      </c>
+      <c r="J94" t="n">
+        <v>0.7038881133020558</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>2.242333333333333</v>
+        <v>0.9318787878787879</v>
       </c>
       <c r="B95" t="n">
-        <v>4862.092484210597</v>
+        <v>4964.271338997541</v>
       </c>
       <c r="C95" t="n">
-        <v>335.978633151851</v>
+        <v>267.7524948451391</v>
       </c>
       <c r="D95" t="n">
-        <v>42.33071173424035</v>
+        <v>41.04066851771798</v>
       </c>
       <c r="E95" t="n">
-        <v>0.9096015481567269</v>
+        <v>0.6953580175672912</v>
       </c>
       <c r="F95" t="n">
-        <v>8.66992478502152</v>
+        <v>8.832557046507141</v>
       </c>
       <c r="G95" t="n">
-        <v>0.5182405362346185</v>
+        <v>0.4394562920562648</v>
       </c>
       <c r="H95" t="n">
-        <v>1.582155750255345e+21</v>
+        <v>4.436716766746465e+20</v>
       </c>
       <c r="I95" t="n">
-        <v>1.442235393625411e+21</v>
+        <v>3.092993849249606e+20</v>
+      </c>
+      <c r="J95" t="n">
+        <v>0.6971357451599872</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>2.266444444444444</v>
+        <v>0.9418989898989898</v>
       </c>
       <c r="B96" t="n">
-        <v>4855.190729227174</v>
+        <v>4963.183091297118</v>
       </c>
       <c r="C96" t="n">
-        <v>333.229999087061</v>
+        <v>264.8925651074281</v>
       </c>
       <c r="D96" t="n">
-        <v>42.30541276676867</v>
+        <v>41.03778504029781</v>
       </c>
       <c r="E96" t="n">
-        <v>0.9047268190990791</v>
+        <v>0.6882324389415098</v>
       </c>
       <c r="F96" t="n">
-        <v>8.659301676192431</v>
+        <v>8.830771486300931</v>
       </c>
       <c r="G96" t="n">
-        <v>0.5118114156897414</v>
+        <v>0.4344795964780693</v>
       </c>
       <c r="H96" t="n">
-        <v>1.540740761207108e+21</v>
+        <v>4.42304769149665e+20</v>
       </c>
       <c r="I96" t="n">
-        <v>1.39692097376219e+21</v>
+        <v>3.051853525169354e+20</v>
+      </c>
+      <c r="J96" t="n">
+        <v>0.6899888353084166</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>2.290555555555556</v>
+        <v>0.9519191919191918</v>
       </c>
       <c r="B97" t="n">
-        <v>4851.848623369023</v>
+        <v>4962.256803255907</v>
       </c>
       <c r="C97" t="n">
-        <v>330.5725296084739</v>
+        <v>261.9917895322917</v>
       </c>
       <c r="D97" t="n">
-        <v>42.27275803865912</v>
+        <v>41.03455586489004</v>
       </c>
       <c r="E97" t="n">
-        <v>0.8987486251263733</v>
+        <v>0.6809499191082158</v>
       </c>
       <c r="F97" t="n">
-        <v>8.654173800147937</v>
+        <v>8.829252620210189</v>
       </c>
       <c r="G97" t="n">
-        <v>0.5066794885605774</v>
+        <v>0.4294837420067614</v>
       </c>
       <c r="H97" t="n">
-        <v>1.490357806595768e+21</v>
+        <v>4.408029632448063e+20</v>
       </c>
       <c r="I97" t="n">
-        <v>1.342296110192294e+21</v>
+        <v>3.009296197372874e+20</v>
+      </c>
+      <c r="J97" t="n">
+        <v>0.6826851106492262</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>2.314666666666667</v>
+        <v>0.9619393939393939</v>
       </c>
       <c r="B98" t="n">
-        <v>4852.48816943881</v>
+        <v>4961.479635122698</v>
       </c>
       <c r="C98" t="n">
-        <v>328.0568327887163</v>
+        <v>259.1416197560064</v>
       </c>
       <c r="D98" t="n">
-        <v>42.23193926560847</v>
+        <v>41.03100130555108</v>
       </c>
       <c r="E98" t="n">
-        <v>0.8916739523275726</v>
+        <v>0.6737529903358779</v>
       </c>
       <c r="F98" t="n">
-        <v>8.65515430558534</v>
+        <v>8.827978931406282</v>
       </c>
       <c r="G98" t="n">
-        <v>0.5030229136286439</v>
+        <v>0.4246141176227647</v>
       </c>
       <c r="H98" t="n">
-        <v>1.430910205137188e+21</v>
+        <v>4.391755207601722e+20</v>
       </c>
       <c r="I98" t="n">
-        <v>1.278612691143311e+21</v>
+        <v>2.966488662536714e+20</v>
+      </c>
+      <c r="J98" t="n">
+        <v>0.6754676711948782</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>2.338777777777778</v>
+        <v>0.9719595959595959</v>
       </c>
       <c r="B99" t="n">
-        <v>4857.541727674715</v>
+        <v>4960.838816937207</v>
       </c>
       <c r="C99" t="n">
-        <v>325.7454273244032</v>
+        <v>256.4354379277085</v>
       </c>
       <c r="D99" t="n">
-        <v>42.1821688538833</v>
+        <v>41.02714157939072</v>
       </c>
       <c r="E99" t="n">
-        <v>0.8835501621568701</v>
+        <v>0.6668893345075033</v>
       </c>
       <c r="F99" t="n">
-        <v>8.662915272128572</v>
+        <v>8.826929069678849</v>
       </c>
       <c r="G99" t="n">
-        <v>0.5010442621401358</v>
+        <v>0.4200189478532232</v>
       </c>
       <c r="H99" t="n">
-        <v>1.362657207595209e+21</v>
+        <v>4.374316631475023e+20</v>
       </c>
       <c r="I99" t="n">
-        <v>1.206552821940407e+21</v>
+        <v>2.924601508810477e+20</v>
+      </c>
+      <c r="J99" t="n">
+        <v>0.668584776823597</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>2.362888888888889</v>
+        <v>0.981979797979798</v>
       </c>
       <c r="B100" t="n">
-        <v>4867.442135009845</v>
+        <v>4960.30195152525</v>
       </c>
       <c r="C100" t="n">
-        <v>323.7133712453564</v>
+        <v>253.9324664560222</v>
       </c>
       <c r="D100" t="n">
-        <v>42.12271318312796</v>
+        <v>41.02303225817941</v>
       </c>
       <c r="E100" t="n">
-        <v>0.8744701855304936</v>
+        <v>0.6605230311338914</v>
       </c>
       <c r="F100" t="n">
-        <v>8.678190238942367</v>
+        <v>8.82604990908067</v>
       </c>
       <c r="G100" t="n">
-        <v>0.5009732257015644</v>
+        <v>0.415785697232419</v>
       </c>
       <c r="H100" t="n">
-        <v>1.286264985395657e+21</v>
+        <v>4.355944147817773e+20</v>
       </c>
       <c r="I100" t="n">
-        <v>1.127248619118938e+21</v>
+        <v>2.884509783884996e+20</v>
+      </c>
+      <c r="J100" t="n">
+        <v>0.6622008193860952</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
-        <v>2.387</v>
+        <v>0.992</v>
       </c>
       <c r="B101" t="n">
-        <v>4882.611188022177</v>
+        <v>4959.749923820569</v>
       </c>
       <c r="C101" t="n">
-        <v>322.0481584443534</v>
+        <v>251.5350316070949</v>
       </c>
       <c r="D101" t="n">
-        <v>42.05292957855509</v>
+        <v>41.0188851166622</v>
       </c>
       <c r="E101" t="n">
-        <v>0.8645746532439412</v>
+        <v>0.6544325355560767</v>
       </c>
       <c r="F101" t="n">
-        <v>8.701775565522821</v>
+        <v>8.825146164074669</v>
       </c>
       <c r="G101" t="n">
-        <v>0.5030687951497622</v>
+        <v>0.4117241230186885</v>
       </c>
       <c r="H101" t="n">
-        <v>1.202825217638963e+21</v>
+        <v>4.337472655942551e+20</v>
       </c>
       <c r="I101" t="n">
-        <v>1.042254527842511e+21</v>
+        <v>2.845787000086306e+20</v>
+      </c>
+      <c r="J101" t="n">
+        <v>0.656093358003638</v>
       </c>
     </row>
   </sheetData>

</xml_diff>